<commit_message>
docs: record preparation verification and push evidence
</commit_message>
<xml_diff>
--- a/Mstar-Property-Task-Tracker.xlsx
+++ b/Mstar-Property-Task-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="1" r:id="R257da747b9b0469a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="2" r:id="R8e699934dc034eab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" r:id="R51d779ea1f6944fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Done" sheetId="4" r:id="R6aefc2579bcc4eec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="5" r:id="Rc296b3c00bbf44fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not started" sheetId="6" r:id="R0be3e7a7d1244657"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="1" r:id="R40fd5b7816544953"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="2" r:id="R50be22aacf4c462e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" r:id="R8a01334b2115450d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Done" sheetId="4" r:id="Rbf35a2d2342b4ba7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="5" r:id="R60459019ad5a44ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not started" sheetId="6" r:id="R56058d6d2a254686"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5546,7 +5546,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a2543aef12142d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R304e6b669a70445c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6657,13 +6657,14 @@
         <x:v>PASS: source inventory, prototype JS syntax, immutable-source hashes, six-sheet IDs and synchronized views. NOT RUN: real-app browser/DB tests; application absent.</x:v>
       </x:c>
       <x:c r="K39" s="44" t="str">
-        <x:v>Local main connected to empty origin. Commit/push recorded in progress.md and final report.</x:v>
+        <x:v>cd897da pushed to origin/main successfully on 2026-10-09. This records the preceding preparation commit; final report identifies the latest verification commit.</x:v>
       </x:c>
       <x:c r="L39" s="44" t="str">
-        <x:v>Preparation files mirrored to live/. SHA-256 verification recorded in testing.md. No deployable application exists.</x:v>
+        <x:v>17 allowlisted preparation files match live by SHA-256. No deployable app exists. No secrets, .git, dependencies or caches copied.</x:v>
       </x:c>
       <x:c r="M39" s="44" t="str">
-        <x:v>2026-10-09: Preparation recorded. Pending real-app/DB tests and localhost verification. Preserve this ID for subsequent updates.</x:v>
+        <x:v>2026-10-09: Preparation recorded. Pending real-app/DB tests and localhost verification. Preserve this ID for subsequent updates.
+2026-10-09: cd897da pushed. Six sheets rendered; 81 IDs verified; 79 original IDs preserved. Preparation mirror hashes pass. R01 remains Pending for real-app/DB tests and localhost verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="150" customHeight="1">
@@ -10408,7 +10409,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3153e067c4b549a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6726c2883a704b4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14681,7 +14682,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbca62864724a4ddf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44035d5ab3434e21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19211,13 +19212,14 @@
         <x:v>PASS: source inventory, prototype JS syntax, immutable-source hashes, six-sheet IDs and synchronized views. NOT RUN: real-app browser/DB tests; application absent.</x:v>
       </x:c>
       <x:c r="K16" s="44" t="str">
-        <x:v>Local main connected to empty origin. Commit/push recorded in progress.md and final report.</x:v>
+        <x:v>cd897da pushed to origin/main successfully on 2026-10-09. This records the preceding preparation commit; final report identifies the latest verification commit.</x:v>
       </x:c>
       <x:c r="L16" s="44" t="str">
-        <x:v>Preparation files mirrored to live/. SHA-256 verification recorded in testing.md. No deployable application exists.</x:v>
+        <x:v>17 allowlisted preparation files match live by SHA-256. No deployable app exists. No secrets, .git, dependencies or caches copied.</x:v>
       </x:c>
       <x:c r="M16" s="44" t="str">
-        <x:v>2026-10-09: Preparation recorded. Pending real-app/DB tests and localhost verification. Preserve this ID for subsequent updates.</x:v>
+        <x:v>2026-10-09: Preparation recorded. Pending real-app/DB tests and localhost verification. Preserve this ID for subsequent updates.
+2026-10-09: cd897da pushed. Six sheets rendered; 81 IDs verified; 79 original IDs preserved. Preparation mirror hashes pass. R01 remains Pending for real-app/DB tests and localhost verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -23115,7 +23117,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d820f6c8e1846aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79ad2f6503194b1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28700,7 +28702,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e67604f301a47f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bebc63bbbba49e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record owner branding currency pricing and chat decisions
</commit_message>
<xml_diff>
--- a/Mstar-Property-Task-Tracker.xlsx
+++ b/Mstar-Property-Task-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="1" r:id="R40fd5b7816544953"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="2" r:id="R50be22aacf4c462e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" r:id="R8a01334b2115450d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Done" sheetId="4" r:id="Rbf35a2d2342b4ba7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="5" r:id="R60459019ad5a44ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not started" sheetId="6" r:id="R56058d6d2a254686"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="1" r:id="R9c82dfab0b064f86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="2" r:id="R94fc5426d11e4030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" r:id="R868c1daef7894273"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Done" sheetId="4" r:id="Rdce67be8736a42d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="5" r:id="R4b1504229c424cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not started" sheetId="6" r:id="R641e1a803ce443d4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="46">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -191,6 +191,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -765,63 +768,85 @@
         <x:v>History</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="26" customHeight="1">
-      <x:c r="A6" s="34" t="str">
+    <x:row r="6" ht="200" customHeight="1">
+      <x:c r="A6" s="46" t="str">
         <x:v>F02</x:v>
       </x:c>
-      <x:c r="B6" s="32" t="str">
+      <x:c r="B6" s="44" t="str">
         <x:v>Decision · Branding</x:v>
       </x:c>
-      <x:c r="C6" s="32" t="str">
+      <x:c r="C6" s="44" t="str">
         <x:v>Owner approves gold / blue / teal / coral accent</x:v>
       </x:c>
-      <x:c r="D6" s="32" t="str">
+      <x:c r="D6" s="44" t="str">
         <x:v>Frontend</x:v>
       </x:c>
-      <x:c r="E6" s="32" t="str">
+      <x:c r="E6" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F6" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #1: accent not finalized</x:v>
-      </x:c>
-      <x:c r="G6" s="32" t="str">
-        <x:v>Owner: approve accent</x:v>
-      </x:c>
-      <x:c r="H6" s="41"/>
-      <x:c r="I6" s="41"/>
-      <x:c r="J6" s="42"/>
-      <x:c r="K6" s="42"/>
-      <x:c r="L6" s="42"/>
-      <x:c r="M6" s="42"/>
-    </x:row>
-    <x:row r="7" ht="26" customHeight="1">
-      <x:c r="A7" s="34" t="str">
+      <x:c r="F6" s="44" t="str">
+        <x:v>Owner selected approved wireframe colours: default gold #f2a91a and associated V3 tokens. Choice recorded; implementation/runtime completion gates remain pending.</x:v>
+      </x:c>
+      <x:c r="G6" s="44" t="str">
+        <x:v>Codex: use exact wireframe tokens when building the foundation.</x:v>
+      </x:c>
+      <x:c r="H6" s="45"/>
+      <x:c r="I6" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J6" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K6" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L6" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M6" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #1: accent not finalized
+2026-10-09 owner update: Owner selected approved wireframe colours: default gold #f2a91a and associated V3 tokens. Choice recorded; implementation/runtime completion gates remain pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="200" customHeight="1">
+      <x:c r="A7" s="46" t="str">
         <x:v>F03</x:v>
       </x:c>
-      <x:c r="B7" s="32" t="str">
+      <x:c r="B7" s="44" t="str">
         <x:v>Decision · Branding</x:v>
       </x:c>
-      <x:c r="C7" s="32" t="str">
+      <x:c r="C7" s="44" t="str">
         <x:v>Provide final crest or horizontal logo for white header</x:v>
       </x:c>
-      <x:c r="D7" s="32" t="str">
+      <x:c r="D7" s="44" t="str">
         <x:v>Frontend</x:v>
       </x:c>
-      <x:c r="E7" s="32" t="str">
+      <x:c r="E7" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F7" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #2 and §11: logo source needed</x:v>
-      </x:c>
-      <x:c r="G7" s="32" t="str">
-        <x:v>Owner/designer: supply approved logo asset</x:v>
-      </x:c>
-      <x:c r="H7" s="41"/>
-      <x:c r="I7" s="41"/>
-      <x:c r="J7" s="42"/>
-      <x:c r="K7" s="42"/>
-      <x:c r="L7" s="42"/>
-      <x:c r="M7" s="42"/>
+      <x:c r="F7" s="44" t="str">
+        <x:v>Owner will add header logo later. Final asset/version deferred. Temporary approved crest can be used during foundation work.</x:v>
+      </x:c>
+      <x:c r="G7" s="44" t="str">
+        <x:v>Owner/designer: supply final header logo later.</x:v>
+      </x:c>
+      <x:c r="H7" s="45"/>
+      <x:c r="I7" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J7" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K7" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L7" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M7" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #2 and §11: logo source needed
+2026-10-09 owner update: Owner will add header logo later. Final asset/version deferred. Temporary approved crest can be used during foundation work.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="26" customHeight="1">
       <x:c r="A8" s="34" t="str">
@@ -5546,7 +5571,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R304e6b669a70445c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a77b8b9ce154b76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5668,34 +5693,45 @@
         <x:v>History</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="26" customHeight="1">
-      <x:c r="A6" s="34" t="str">
+    <x:row r="6" ht="200" customHeight="1">
+      <x:c r="A6" s="46" t="str">
         <x:v>B09</x:v>
       </x:c>
-      <x:c r="B6" s="32" t="str">
+      <x:c r="B6" s="44" t="str">
         <x:v>Decision · Map</x:v>
       </x:c>
-      <x:c r="C6" s="32" t="str">
+      <x:c r="C6" s="44" t="str">
         <x:v>Approve Google Maps Platform or Longdo Map</x:v>
       </x:c>
-      <x:c r="D6" s="32" t="str">
+      <x:c r="D6" s="44" t="str">
         <x:v>Backend</x:v>
       </x:c>
-      <x:c r="E6" s="32" t="str">
+      <x:c r="E6" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F6" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #8: map provider not selected</x:v>
-      </x:c>
-      <x:c r="G6" s="32" t="str">
-        <x:v>Owner: select map provider and API account</x:v>
-      </x:c>
-      <x:c r="H6" s="41"/>
-      <x:c r="I6" s="41"/>
-      <x:c r="J6" s="42"/>
-      <x:c r="K6" s="42"/>
-      <x:c r="L6" s="42"/>
-      <x:c r="M6" s="42"/>
+      <x:c r="F6" s="44" t="str">
+        <x:v>Owner requests free open-source mapping for now. Specific library and tile/nearby provider remain undecided.</x:v>
+      </x:c>
+      <x:c r="G6" s="44" t="str">
+        <x:v>Codex: evaluate free open-source mapping before map step; confirm provider and usage policy.</x:v>
+      </x:c>
+      <x:c r="H6" s="45"/>
+      <x:c r="I6" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J6" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K6" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L6" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M6" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #8: map provider not selected
+2026-10-09 owner update: Owner requests free open-source mapping for now. Specific library and tile/nearby provider remain undecided.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="26" customHeight="1">
       <x:c r="A7" s="34" t="str">
@@ -5726,34 +5762,45 @@
       <x:c r="L7" s="42"/>
       <x:c r="M7" s="42"/>
     </x:row>
-    <x:row r="8" ht="26" customHeight="1">
-      <x:c r="A8" s="34" t="str">
+    <x:row r="8" ht="200" customHeight="1">
+      <x:c r="A8" s="46" t="str">
         <x:v>B18</x:v>
       </x:c>
-      <x:c r="B8" s="32" t="str">
+      <x:c r="B8" s="44" t="str">
         <x:v>Decision · Chat</x:v>
       </x:c>
-      <x:c r="C8" s="32" t="str">
+      <x:c r="C8" s="44" t="str">
         <x:v>Approve company-wide versus per-agent LINE/WhatsApp IDs</x:v>
       </x:c>
-      <x:c r="D8" s="32" t="str">
+      <x:c r="D8" s="44" t="str">
         <x:v>Backend</x:v>
       </x:c>
-      <x:c r="E8" s="32" t="str">
+      <x:c r="E8" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F8" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #4 unresolved</x:v>
-      </x:c>
-      <x:c r="G8" s="32" t="str">
-        <x:v>Owner: confirm IDs/numbers</x:v>
-      </x:c>
-      <x:c r="H8" s="41"/>
-      <x:c r="I8" s="41"/>
-      <x:c r="J8" s="42"/>
-      <x:c r="K8" s="42"/>
-      <x:c r="L8" s="42"/>
-      <x:c r="M8" s="42"/>
+      <x:c r="F8" s="44" t="str">
+        <x:v>Owner requests LINE and WhatsApp buttons first. Actual contacts and company versus per-agent routing remain unresolved.</x:v>
+      </x:c>
+      <x:c r="G8" s="44" t="str">
+        <x:v>Codex: create approved buttons first in foundation; owner: provide contacts before integration.</x:v>
+      </x:c>
+      <x:c r="H8" s="45"/>
+      <x:c r="I8" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J8" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K8" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L8" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M8" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #4 unresolved
+2026-10-09 owner update: Owner requests LINE and WhatsApp buttons first. Actual contacts and company versus per-agent routing remain unresolved.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
       <x:c r="A9" s="34" t="str">
@@ -5784,63 +5831,85 @@
       <x:c r="L9" s="42"/>
       <x:c r="M9" s="42"/>
     </x:row>
-    <x:row r="10" ht="26" customHeight="1">
-      <x:c r="A10" s="34" t="str">
+    <x:row r="10" ht="200" customHeight="1">
+      <x:c r="A10" s="46" t="str">
         <x:v>B28</x:v>
       </x:c>
-      <x:c r="B10" s="32" t="str">
+      <x:c r="B10" s="44" t="str">
         <x:v>Decision · Currency</x:v>
       </x:c>
-      <x:c r="C10" s="32" t="str">
+      <x:c r="C10" s="44" t="str">
         <x:v>Approve THB only versus optional approximate FX display</x:v>
       </x:c>
-      <x:c r="D10" s="32" t="str">
+      <x:c r="D10" s="44" t="str">
         <x:v>Backend</x:v>
       </x:c>
-      <x:c r="E10" s="32" t="str">
+      <x:c r="E10" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F10" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #6 unresolved</x:v>
-      </x:c>
-      <x:c r="G10" s="32" t="str">
-        <x:v>Owner: approve currency policy</x:v>
-      </x:c>
-      <x:c r="H10" s="41"/>
-      <x:c r="I10" s="41"/>
-      <x:c r="J10" s="42"/>
-      <x:c r="K10" s="42"/>
-      <x:c r="L10" s="42"/>
-      <x:c r="M10" s="42"/>
-    </x:row>
-    <x:row r="11" ht="26" customHeight="1">
-      <x:c r="A11" s="34" t="str">
+      <x:c r="F10" s="44" t="str">
+        <x:v>Owner selected USD (US dollars) and THB. Store THB base; display approximate USD using daily rates. Rate source not selected; code not built.</x:v>
+      </x:c>
+      <x:c r="G10" s="44" t="str">
+        <x:v>Codex: implement USD/THB during authorized currency work; confirm rate source.</x:v>
+      </x:c>
+      <x:c r="H10" s="45"/>
+      <x:c r="I10" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J10" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K10" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L10" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M10" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #6 unresolved
+2026-10-09 owner update: Owner selected USD (US dollars) and THB. Store THB base; display approximate USD using daily rates. Rate source not selected; code not built.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="200" customHeight="1">
+      <x:c r="A11" s="46" t="str">
         <x:v>B29</x:v>
       </x:c>
-      <x:c r="B11" s="32" t="str">
+      <x:c r="B11" s="44" t="str">
         <x:v>Decision · Projects</x:v>
       </x:c>
-      <x:c r="C11" s="32" t="str">
+      <x:c r="C11" s="44" t="str">
         <x:v>Approve public project prices versus enquiry-only price list</x:v>
       </x:c>
-      <x:c r="D11" s="32" t="str">
+      <x:c r="D11" s="44" t="str">
         <x:v>Backend</x:v>
       </x:c>
-      <x:c r="E11" s="32" t="str">
+      <x:c r="E11" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F11" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #7 unresolved</x:v>
-      </x:c>
-      <x:c r="G11" s="32" t="str">
-        <x:v>Owner: approve project price visibility</x:v>
-      </x:c>
-      <x:c r="H11" s="41"/>
-      <x:c r="I11" s="41"/>
-      <x:c r="J11" s="42"/>
-      <x:c r="K11" s="42"/>
-      <x:c r="L11" s="42"/>
-      <x:c r="M11" s="42"/>
+      <x:c r="F11" s="44" t="str">
+        <x:v>Owner selected both public and contact-gated pricing, chosen by admin per listing/product or project. Choice recorded; implementation pending.</x:v>
+      </x:c>
+      <x:c r="G11" s="44" t="str">
+        <x:v>Codex: add per-record price visibility in authorized backend/admin work after admin wireframe approval.</x:v>
+      </x:c>
+      <x:c r="H11" s="45"/>
+      <x:c r="I11" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J11" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K11" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L11" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M11" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #7 unresolved
+2026-10-09 owner update: Owner selected both public and contact-gated pricing, chosen by admin per listing/product or project. Choice recorded; implementation pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="26" customHeight="1">
       <x:c r="A12" s="34" t="str">
@@ -6625,7 +6694,7 @@
       <x:c r="L38" s="42"/>
       <x:c r="M38" s="42"/>
     </x:row>
-    <x:row r="39" ht="150" customHeight="1">
+    <x:row r="39" ht="200" customHeight="1">
       <x:c r="A39" s="44" t="str">
         <x:v>R01</x:v>
       </x:c>
@@ -6642,10 +6711,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F39" s="44" t="str">
-        <x:v>Documentation and tracker prepared. Git/live hashes checked. No application, health API, admin or project PostgreSQL configuration exists. Browser file navigation is blocked. G4/G5 remain pending.</x:v>
+        <x:v>Owner choices documented and tracker updated. Foundation remains unbuilt; no app, PostgreSQL configuration or verified localhost URLs. Runtime gates remain pending.</x:v>
       </x:c>
       <x:c r="G39" s="44" t="str">
-        <x:v>Owner: provide Step 1 start prompt and branding choices. Codex: build only authorized foundation, then test real app.</x:v>
+        <x:v>Owner: start foundation build. Codex: prioritize approved LINE/WhatsApp buttons, then finish authorized foundation and test.</x:v>
       </x:c>
       <x:c r="H39" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -6654,17 +6723,18 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J39" s="44" t="str">
-        <x:v>PASS: source inventory, prototype JS syntax, immutable-source hashes, six-sheet IDs and synchronized views. NOT RUN: real-app browser/DB tests; application absent.</x:v>
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
       </x:c>
       <x:c r="K39" s="44" t="str">
-        <x:v>cd897da pushed to origin/main successfully on 2026-10-09. This records the preceding preparation commit; final report identifies the latest verification commit.</x:v>
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
       </x:c>
       <x:c r="L39" s="44" t="str">
-        <x:v>17 allowlisted preparation files match live by SHA-256. No deployable app exists. No secrets, .git, dependencies or caches copied.</x:v>
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
       </x:c>
       <x:c r="M39" s="44" t="str">
         <x:v>2026-10-09: Preparation recorded. Pending real-app/DB tests and localhost verification. Preserve this ID for subsequent updates.
-2026-10-09: cd897da pushed. Six sheets rendered; 81 IDs verified; 79 original IDs preserved. Preparation mirror hashes pass. R01 remains Pending for real-app/DB tests and localhost verification.</x:v>
+2026-10-09: cd897da pushed. Six sheets rendered; 81 IDs verified; 79 original IDs preserved. Preparation mirror hashes pass. R01 remains Pending for real-app/DB tests and localhost verification.
+2026-10-09 owner update: Owner choices documented and tracker updated. Foundation remains unbuilt; no app, PostgreSQL configuration or verified localhost URLs. Runtime gates remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="150" customHeight="1">
@@ -10409,7 +10479,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6726c2883a704b4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc85086fc0e704f3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14682,7 +14752,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44035d5ab3434e21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7eccad8d34364033"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18890,63 +18960,85 @@
         <x:v>History</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="26" customHeight="1">
-      <x:c r="A6" s="34" t="str">
+    <x:row r="6" ht="200" customHeight="1">
+      <x:c r="A6" s="46" t="str">
         <x:v>F02</x:v>
       </x:c>
-      <x:c r="B6" s="32" t="str">
+      <x:c r="B6" s="44" t="str">
         <x:v>Decision · Branding</x:v>
       </x:c>
-      <x:c r="C6" s="32" t="str">
+      <x:c r="C6" s="44" t="str">
         <x:v>Owner approves gold / blue / teal / coral accent</x:v>
       </x:c>
-      <x:c r="D6" s="32" t="str">
+      <x:c r="D6" s="44" t="str">
         <x:v>Frontend</x:v>
       </x:c>
-      <x:c r="E6" s="32" t="str">
+      <x:c r="E6" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F6" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #1: accent not finalized</x:v>
-      </x:c>
-      <x:c r="G6" s="32" t="str">
-        <x:v>Owner: approve accent</x:v>
-      </x:c>
-      <x:c r="H6" s="41"/>
-      <x:c r="I6" s="41"/>
-      <x:c r="J6" s="42"/>
-      <x:c r="K6" s="42"/>
-      <x:c r="L6" s="42"/>
-      <x:c r="M6" s="42"/>
-    </x:row>
-    <x:row r="7" ht="26" customHeight="1">
-      <x:c r="A7" s="34" t="str">
+      <x:c r="F6" s="44" t="str">
+        <x:v>Owner selected approved wireframe colours: default gold #f2a91a and associated V3 tokens. Choice recorded; implementation/runtime completion gates remain pending.</x:v>
+      </x:c>
+      <x:c r="G6" s="44" t="str">
+        <x:v>Codex: use exact wireframe tokens when building the foundation.</x:v>
+      </x:c>
+      <x:c r="H6" s="45"/>
+      <x:c r="I6" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J6" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K6" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L6" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M6" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #1: accent not finalized
+2026-10-09 owner update: Owner selected approved wireframe colours: default gold #f2a91a and associated V3 tokens. Choice recorded; implementation/runtime completion gates remain pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="200" customHeight="1">
+      <x:c r="A7" s="46" t="str">
         <x:v>F03</x:v>
       </x:c>
-      <x:c r="B7" s="32" t="str">
+      <x:c r="B7" s="44" t="str">
         <x:v>Decision · Branding</x:v>
       </x:c>
-      <x:c r="C7" s="32" t="str">
+      <x:c r="C7" s="44" t="str">
         <x:v>Provide final crest or horizontal logo for white header</x:v>
       </x:c>
-      <x:c r="D7" s="32" t="str">
+      <x:c r="D7" s="44" t="str">
         <x:v>Frontend</x:v>
       </x:c>
-      <x:c r="E7" s="32" t="str">
+      <x:c r="E7" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F7" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #2 and §11: logo source needed</x:v>
-      </x:c>
-      <x:c r="G7" s="32" t="str">
-        <x:v>Owner/designer: supply approved logo asset</x:v>
-      </x:c>
-      <x:c r="H7" s="41"/>
-      <x:c r="I7" s="41"/>
-      <x:c r="J7" s="42"/>
-      <x:c r="K7" s="42"/>
-      <x:c r="L7" s="42"/>
-      <x:c r="M7" s="42"/>
+      <x:c r="F7" s="44" t="str">
+        <x:v>Owner will add header logo later. Final asset/version deferred. Temporary approved crest can be used during foundation work.</x:v>
+      </x:c>
+      <x:c r="G7" s="44" t="str">
+        <x:v>Owner/designer: supply final header logo later.</x:v>
+      </x:c>
+      <x:c r="H7" s="45"/>
+      <x:c r="I7" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J7" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K7" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L7" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M7" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #2 and §11: logo source needed
+2026-10-09 owner update: Owner will add header logo later. Final asset/version deferred. Temporary approved crest can be used during foundation work.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="26" customHeight="1">
       <x:c r="A8" s="34" t="str">
@@ -19006,34 +19098,45 @@
       <x:c r="L9" s="42"/>
       <x:c r="M9" s="42"/>
     </x:row>
-    <x:row r="10" ht="26" customHeight="1">
-      <x:c r="A10" s="34" t="str">
+    <x:row r="10" ht="200" customHeight="1">
+      <x:c r="A10" s="46" t="str">
         <x:v>B09</x:v>
       </x:c>
-      <x:c r="B10" s="32" t="str">
+      <x:c r="B10" s="44" t="str">
         <x:v>Decision · Map</x:v>
       </x:c>
-      <x:c r="C10" s="32" t="str">
+      <x:c r="C10" s="44" t="str">
         <x:v>Approve Google Maps Platform or Longdo Map</x:v>
       </x:c>
-      <x:c r="D10" s="32" t="str">
+      <x:c r="D10" s="44" t="str">
         <x:v>Backend</x:v>
       </x:c>
-      <x:c r="E10" s="32" t="str">
+      <x:c r="E10" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F10" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #8: map provider not selected</x:v>
-      </x:c>
-      <x:c r="G10" s="32" t="str">
-        <x:v>Owner: select map provider and API account</x:v>
-      </x:c>
-      <x:c r="H10" s="41"/>
-      <x:c r="I10" s="41"/>
-      <x:c r="J10" s="42"/>
-      <x:c r="K10" s="42"/>
-      <x:c r="L10" s="42"/>
-      <x:c r="M10" s="42"/>
+      <x:c r="F10" s="44" t="str">
+        <x:v>Owner requests free open-source mapping for now. Specific library and tile/nearby provider remain undecided.</x:v>
+      </x:c>
+      <x:c r="G10" s="44" t="str">
+        <x:v>Codex: evaluate free open-source mapping before map step; confirm provider and usage policy.</x:v>
+      </x:c>
+      <x:c r="H10" s="45"/>
+      <x:c r="I10" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J10" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K10" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L10" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M10" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #8: map provider not selected
+2026-10-09 owner update: Owner requests free open-source mapping for now. Specific library and tile/nearby provider remain undecided.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="26" customHeight="1">
       <x:c r="A11" s="34" t="str">
@@ -19064,34 +19167,45 @@
       <x:c r="L11" s="42"/>
       <x:c r="M11" s="42"/>
     </x:row>
-    <x:row r="12" ht="26" customHeight="1">
-      <x:c r="A12" s="34" t="str">
+    <x:row r="12" ht="200" customHeight="1">
+      <x:c r="A12" s="46" t="str">
         <x:v>B18</x:v>
       </x:c>
-      <x:c r="B12" s="32" t="str">
+      <x:c r="B12" s="44" t="str">
         <x:v>Decision · Chat</x:v>
       </x:c>
-      <x:c r="C12" s="32" t="str">
+      <x:c r="C12" s="44" t="str">
         <x:v>Approve company-wide versus per-agent LINE/WhatsApp IDs</x:v>
       </x:c>
-      <x:c r="D12" s="32" t="str">
+      <x:c r="D12" s="44" t="str">
         <x:v>Backend</x:v>
       </x:c>
-      <x:c r="E12" s="32" t="str">
+      <x:c r="E12" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F12" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #4 unresolved</x:v>
-      </x:c>
-      <x:c r="G12" s="32" t="str">
-        <x:v>Owner: confirm IDs/numbers</x:v>
-      </x:c>
-      <x:c r="H12" s="41"/>
-      <x:c r="I12" s="41"/>
-      <x:c r="J12" s="42"/>
-      <x:c r="K12" s="42"/>
-      <x:c r="L12" s="42"/>
-      <x:c r="M12" s="42"/>
+      <x:c r="F12" s="44" t="str">
+        <x:v>Owner requests LINE and WhatsApp buttons first. Actual contacts and company versus per-agent routing remain unresolved.</x:v>
+      </x:c>
+      <x:c r="G12" s="44" t="str">
+        <x:v>Codex: create approved buttons first in foundation; owner: provide contacts before integration.</x:v>
+      </x:c>
+      <x:c r="H12" s="45"/>
+      <x:c r="I12" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J12" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K12" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L12" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M12" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #4 unresolved
+2026-10-09 owner update: Owner requests LINE and WhatsApp buttons first. Actual contacts and company versus per-agent routing remain unresolved.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="26" customHeight="1">
       <x:c r="A13" s="34" t="str">
@@ -19122,65 +19236,87 @@
       <x:c r="L13" s="42"/>
       <x:c r="M13" s="42"/>
     </x:row>
-    <x:row r="14" ht="26" customHeight="1">
-      <x:c r="A14" s="34" t="str">
+    <x:row r="14" ht="200" customHeight="1">
+      <x:c r="A14" s="46" t="str">
         <x:v>B28</x:v>
       </x:c>
-      <x:c r="B14" s="32" t="str">
+      <x:c r="B14" s="44" t="str">
         <x:v>Decision · Currency</x:v>
       </x:c>
-      <x:c r="C14" s="32" t="str">
+      <x:c r="C14" s="44" t="str">
         <x:v>Approve THB only versus optional approximate FX display</x:v>
       </x:c>
-      <x:c r="D14" s="32" t="str">
+      <x:c r="D14" s="44" t="str">
         <x:v>Backend</x:v>
       </x:c>
-      <x:c r="E14" s="32" t="str">
+      <x:c r="E14" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F14" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #6 unresolved</x:v>
-      </x:c>
-      <x:c r="G14" s="32" t="str">
-        <x:v>Owner: approve currency policy</x:v>
-      </x:c>
-      <x:c r="H14" s="41"/>
-      <x:c r="I14" s="41"/>
-      <x:c r="J14" s="42"/>
-      <x:c r="K14" s="42"/>
-      <x:c r="L14" s="42"/>
-      <x:c r="M14" s="42"/>
-    </x:row>
-    <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="34" t="str">
+      <x:c r="F14" s="44" t="str">
+        <x:v>Owner selected USD (US dollars) and THB. Store THB base; display approximate USD using daily rates. Rate source not selected; code not built.</x:v>
+      </x:c>
+      <x:c r="G14" s="44" t="str">
+        <x:v>Codex: implement USD/THB during authorized currency work; confirm rate source.</x:v>
+      </x:c>
+      <x:c r="H14" s="45"/>
+      <x:c r="I14" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J14" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K14" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L14" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M14" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #6 unresolved
+2026-10-09 owner update: Owner selected USD (US dollars) and THB. Store THB base; display approximate USD using daily rates. Rate source not selected; code not built.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="200" customHeight="1">
+      <x:c r="A15" s="46" t="str">
         <x:v>B29</x:v>
       </x:c>
-      <x:c r="B15" s="32" t="str">
+      <x:c r="B15" s="44" t="str">
         <x:v>Decision · Projects</x:v>
       </x:c>
-      <x:c r="C15" s="32" t="str">
+      <x:c r="C15" s="44" t="str">
         <x:v>Approve public project prices versus enquiry-only price list</x:v>
       </x:c>
-      <x:c r="D15" s="32" t="str">
+      <x:c r="D15" s="44" t="str">
         <x:v>Backend</x:v>
       </x:c>
-      <x:c r="E15" s="32" t="str">
+      <x:c r="E15" s="44" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="F15" s="32" t="str">
-        <x:v>BUILD-SPEC §12 #7 unresolved</x:v>
-      </x:c>
-      <x:c r="G15" s="32" t="str">
-        <x:v>Owner: approve project price visibility</x:v>
-      </x:c>
-      <x:c r="H15" s="41"/>
-      <x:c r="I15" s="41"/>
-      <x:c r="J15" s="42"/>
-      <x:c r="K15" s="42"/>
-      <x:c r="L15" s="42"/>
-      <x:c r="M15" s="42"/>
-    </x:row>
-    <x:row r="16" ht="150" customHeight="1">
+      <x:c r="F15" s="44" t="str">
+        <x:v>Owner selected both public and contact-gated pricing, chosen by admin per listing/product or project. Choice recorded; implementation pending.</x:v>
+      </x:c>
+      <x:c r="G15" s="44" t="str">
+        <x:v>Codex: add per-record price visibility in authorized backend/admin work after admin wireframe approval.</x:v>
+      </x:c>
+      <x:c r="H15" s="45"/>
+      <x:c r="I15" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J15" s="44" t="str">
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+      </x:c>
+      <x:c r="K15" s="44" t="str">
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+      </x:c>
+      <x:c r="L15" s="44" t="str">
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+      </x:c>
+      <x:c r="M15" s="44" t="str">
+        <x:v>Original planning evidence: BUILD-SPEC §12 #7 unresolved
+2026-10-09 owner update: Owner selected both public and contact-gated pricing, chosen by admin per listing/product or project. Choice recorded; implementation pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="200" customHeight="1">
       <x:c r="A16" s="44" t="str">
         <x:v>R01</x:v>
       </x:c>
@@ -19197,10 +19333,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F16" s="44" t="str">
-        <x:v>Documentation and tracker prepared. Git/live hashes checked. No application, health API, admin or project PostgreSQL configuration exists. Browser file navigation is blocked. G4/G5 remain pending.</x:v>
+        <x:v>Owner choices documented and tracker updated. Foundation remains unbuilt; no app, PostgreSQL configuration or verified localhost URLs. Runtime gates remain pending.</x:v>
       </x:c>
       <x:c r="G16" s="44" t="str">
-        <x:v>Owner: provide Step 1 start prompt and branding choices. Codex: build only authorized foundation, then test real app.</x:v>
+        <x:v>Owner: start foundation build. Codex: prioritize approved LINE/WhatsApp buttons, then finish authorized foundation and test.</x:v>
       </x:c>
       <x:c r="H16" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -19209,17 +19345,18 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J16" s="44" t="str">
-        <x:v>PASS: source inventory, prototype JS syntax, immutable-source hashes, six-sheet IDs and synchronized views. NOT RUN: real-app browser/DB tests; application absent.</x:v>
+        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
       </x:c>
       <x:c r="K16" s="44" t="str">
-        <x:v>cd897da pushed to origin/main successfully on 2026-10-09. This records the preceding preparation commit; final report identifies the latest verification commit.</x:v>
+        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
       </x:c>
       <x:c r="L16" s="44" t="str">
-        <x:v>17 allowlisted preparation files match live by SHA-256. No deployable app exists. No secrets, .git, dependencies or caches copied.</x:v>
+        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
       </x:c>
       <x:c r="M16" s="44" t="str">
         <x:v>2026-10-09: Preparation recorded. Pending real-app/DB tests and localhost verification. Preserve this ID for subsequent updates.
-2026-10-09: cd897da pushed. Six sheets rendered; 81 IDs verified; 79 original IDs preserved. Preparation mirror hashes pass. R01 remains Pending for real-app/DB tests and localhost verification.</x:v>
+2026-10-09: cd897da pushed. Six sheets rendered; 81 IDs verified; 79 original IDs preserved. Preparation mirror hashes pass. R01 remains Pending for real-app/DB tests and localhost verification.
+2026-10-09 owner update: Owner choices documented and tracker updated. Foundation remains unbuilt; no app, PostgreSQL configuration or verified localhost URLs. Runtime gates remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -23117,7 +23254,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79ad2f6503194b1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06f0001341ca4694"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28702,7 +28839,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bebc63bbbba49e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb27453f98bb54861"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: adopt V5 stage guide and revised approved references
</commit_message>
<xml_diff>
--- a/Mstar-Property-Task-Tracker.xlsx
+++ b/Mstar-Property-Task-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="1" r:id="R7b765efbff6245ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="2" r:id="R7334d51d33cd4af8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" r:id="Rc7825516e6a24465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Done" sheetId="4" r:id="R918bc54d48a54859"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="5" r:id="Re3b9a372d07f4f19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not started" sheetId="6" r:id="Rc9aa087cd88842ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="1" r:id="R4a40b80151914e17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="2" r:id="R649c040592ee4b5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" r:id="Ra0cb1649582144db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Done" sheetId="4" r:id="R351d6b6b298b4723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="5" r:id="R4e7644ae36de49bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not started" sheetId="6" r:id="Rd670fa657f854d60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -683,7 +683,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Foundation implemented, Pending runtime gates. 81 permanent IDs; append history. Port 3000 closed on owner request. Category tabs mirror open tasks; status tabs canonical.</x:v>
+        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -1122,7 +1122,7 @@
 2026-10-09 foundation: Thai/English routes, Accept-Language and explicit preference cookies implemented. Redirect checks passed. Four browser preference/search flows failed before closure; Host-based origin fix compiles but remains untested in browser. Owner requested localhost closure; do not reopen automatically.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="26" customHeight="1">
+    <x:row r="15" ht="250" customHeight="1">
       <x:c r="A15" s="46" t="str">
         <x:v>F08</x:v>
       </x:c>
@@ -1130,7 +1130,7 @@
         <x:v>Step 3 · Cards</x:v>
       </x:c>
       <x:c r="C15" s="44" t="str">
-        <x:v>4:3 cards, photo galleries, save heart, badges and type-specific facts</x:v>
+        <x:v>Realtor-style 3:2 listing cards, photo controls, bottom-right save heart, facts/address and Contact agent dialog trigger</x:v>
       </x:c>
       <x:c r="D15" s="44" t="str">
         <x:v>Frontend</x:v>
@@ -1139,17 +1139,28 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="F15" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
+        <x:v>V5 Step 3 and revised BUILD-SPEC 4.3 replace the older 4:3 card plan. One reusable card across homepage/results/Saved. Not implemented; requires Step 2 Done.</x:v>
       </x:c>
       <x:c r="G15" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
+        <x:v>Codex: build revised card only under Step 3 authorization, after the real database step.</x:v>
       </x:c>
       <x:c r="H15" s="45"/>
-      <x:c r="I15" s="45"/>
-      <x:c r="J15" s="44"/>
-      <x:c r="K15" s="44"/>
-      <x:c r="L15" s="44"/>
-      <x:c r="M15" s="44"/>
+      <x:c r="I15" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J15" s="44" t="str">
+        <x:v>Documentation/planning update only. No application tests run at owner request. Existing runtime test results remain in prior history. Workbook/source/mirror checks performed.</x:v>
+      </x:c>
+      <x:c r="K15" s="44" t="str">
+        <x:v>Preceding foundation commit 604c62e pushed. V5 adoption commit/push verified at finalization; final report provides hash.</x:v>
+      </x:c>
+      <x:c r="L15" s="44" t="str">
+        <x:v>Baseline live files compared with Git before synchronization; revised guide/source/docs/tracker synchronized only after divergence checks.</x:v>
+      </x:c>
+      <x:c r="M15" s="44" t="str">
+        <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
+2026-10-09 V5 adoption: V5 Step 3 and revised BUILD-SPEC 4.3 replace the older 4:3 card plan. One reusable card across homepage/results/Saved. Not implemented; requires Step 2 Done.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="26" customHeight="1">
       <x:c r="A16" s="46" t="str">
@@ -1499,7 +1510,7 @@
       <x:c r="L27" s="44"/>
       <x:c r="M27" s="44"/>
     </x:row>
-    <x:row r="28" ht="26" customHeight="1">
+    <x:row r="28" ht="250" customHeight="1">
       <x:c r="A28" s="46" t="str">
         <x:v>F21</x:v>
       </x:c>
@@ -1507,7 +1518,7 @@
         <x:v>Step 6 · Contact</x:v>
       </x:c>
       <x:c r="C28" s="44" t="str">
-        <x:v>Desktop sticky enquiry box and phone sticky action bar</x:v>
+        <x:v>Shared agent enquiry form, card Contact agent dialog, desktop sticky box and phone contact bar</x:v>
       </x:c>
       <x:c r="D28" s="44" t="str">
         <x:v>Frontend</x:v>
@@ -1516,17 +1527,28 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="F28" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
+        <x:v>V5 Step 6 wires the card dialog and property form through one component/action. No implementation started; destinations still unresolved.</x:v>
       </x:c>
       <x:c r="G28" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
+        <x:v>Owner: provide routing/contacts. Codex: implement only under Step 6 authorization.</x:v>
       </x:c>
       <x:c r="H28" s="45"/>
-      <x:c r="I28" s="45"/>
-      <x:c r="J28" s="44"/>
-      <x:c r="K28" s="44"/>
-      <x:c r="L28" s="44"/>
-      <x:c r="M28" s="44"/>
+      <x:c r="I28" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J28" s="44" t="str">
+        <x:v>Documentation/planning update only. No application tests run at owner request. Existing runtime test results remain in prior history. Workbook/source/mirror checks performed.</x:v>
+      </x:c>
+      <x:c r="K28" s="44" t="str">
+        <x:v>Preceding foundation commit 604c62e pushed. V5 adoption commit/push verified at finalization; final report provides hash.</x:v>
+      </x:c>
+      <x:c r="L28" s="44" t="str">
+        <x:v>Baseline live files compared with Git before synchronization; revised guide/source/docs/tracker synchronized only after divergence checks.</x:v>
+      </x:c>
+      <x:c r="M28" s="44" t="str">
+        <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
+2026-10-09 V5 adoption: V5 Step 6 wires the card dialog and property form through one component/action. No implementation started; destinations still unresolved.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="26" customHeight="1">
       <x:c r="A29" s="46" t="str">
@@ -1615,7 +1637,7 @@
       <x:c r="L31" s="44"/>
       <x:c r="M31" s="44"/>
     </x:row>
-    <x:row r="32" ht="26" customHeight="1">
+    <x:row r="32" ht="250" customHeight="1">
       <x:c r="A32" s="46" t="str">
         <x:v>F25</x:v>
       </x:c>
@@ -1623,7 +1645,7 @@
         <x:v>Step 7 · Home</x:v>
       </x:c>
       <x:c r="C32" s="44" t="str">
-        <x:v>Featured homes, regions with accurate listing counts</x:v>
+        <x:v>Homes for you carousel directly below search; regions with real listing counts</x:v>
       </x:c>
       <x:c r="D32" s="44" t="str">
         <x:v>Frontend</x:v>
@@ -1632,17 +1654,28 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="F32" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
+        <x:v>V5 Step 7 uses Step 3 cards: five tabs, arrows, See all, 3/2/1.1 visible cards, swipe/scroll-snap, featured first then newest, up to 12 per tab. Not implemented.</x:v>
       </x:c>
       <x:c r="G32" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
+        <x:v>Codex: implement approved home-page.html only under Step 7 authorization.</x:v>
       </x:c>
       <x:c r="H32" s="45"/>
-      <x:c r="I32" s="45"/>
-      <x:c r="J32" s="44"/>
-      <x:c r="K32" s="44"/>
-      <x:c r="L32" s="44"/>
-      <x:c r="M32" s="44"/>
+      <x:c r="I32" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J32" s="44" t="str">
+        <x:v>Documentation/planning update only. No application tests run at owner request. Existing runtime test results remain in prior history. Workbook/source/mirror checks performed.</x:v>
+      </x:c>
+      <x:c r="K32" s="44" t="str">
+        <x:v>Preceding foundation commit 604c62e pushed. V5 adoption commit/push verified at finalization; final report provides hash.</x:v>
+      </x:c>
+      <x:c r="L32" s="44" t="str">
+        <x:v>Baseline live files compared with Git before synchronization; revised guide/source/docs/tracker synchronized only after divergence checks.</x:v>
+      </x:c>
+      <x:c r="M32" s="44" t="str">
+        <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
+2026-10-09 V5 adoption: V5 Step 7 uses Step 3 cards: five tabs, arrows, See all, 3/2/1.1 visible cards, swipe/scroll-snap, featured first then newest, up to 12 per tab. Not implemented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="26" customHeight="1">
       <x:c r="A33" s="46" t="str">
@@ -8841,7 +8874,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17602caa8f8b42fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R009d4f61af814f26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8878,7 +8911,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Foundation implemented, Pending runtime gates. 81 permanent IDs; append history. Port 3000 closed on owner request. Category tabs mirror open tasks; status tabs canonical.</x:v>
+        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -9201,10 +9234,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F12" s="44" t="str">
-        <x:v>Preparation and foundation implemented; docs/tracker/source mirror updated. Build passes; 12/16 browser/API tests passed before owner-requested closure. Four preference/search flows need retesting after fixes; PostgreSQL is unconfigured; port 3000 is closed.</x:v>
+        <x:v>V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.</x:v>
       </x:c>
       <x:c r="G12" s="44" t="str">
-        <x:v>Codex: stop before Step 2. Retest only when owner opens localhost; verify real PostgreSQL.</x:v>
+        <x:v>Owner: supply the next stage prompt or authorize deferred tests. Codex: follow V5 one stage at a time; do not automatically advance.</x:v>
       </x:c>
       <x:c r="H12" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -9213,19 +9246,20 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J12" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>Documentation/planning update only. No application tests run at owner request. Existing runtime test results remain in prior history. Workbook/source/mirror checks performed.</x:v>
       </x:c>
       <x:c r="K12" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding foundation commit 604c62e pushed. V5 adoption commit/push verified at finalization; final report provides hash.</x:v>
       </x:c>
       <x:c r="L12" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>Baseline live files compared with Git before synchronization; revised guide/source/docs/tracker synchronized only after divergence checks.</x:v>
       </x:c>
       <x:c r="M12" s="44" t="str">
         <x:v>2026-10-09: Preparation recorded. Pending real-app/DB tests and localhost verification. Preserve this ID for subsequent updates.
 2026-10-09: cd897da pushed. Six sheets rendered; 81 IDs verified; 79 original IDs preserved. Preparation mirror hashes pass. R01 remains Pending for real-app/DB tests and localhost verification.
 2026-10-09 owner update: Owner choices documented and tracker updated. Foundation remains unbuilt; no app, PostgreSQL configuration or verified localhost URLs. Runtime gates remain pending.
-2026-10-09 foundation: Preparation and foundation implemented; docs/tracker/source mirror updated. Build passes; 12/16 browser/API tests passed before owner-requested closure. Four preference/search flows need retesting after fixes; PostgreSQL is unconfigured; port 3000 is closed. Owner requested localhost closure; do not reopen automatically.</x:v>
+2026-10-09 foundation: Preparation and foundation implemented; docs/tracker/source mirror updated. Build passes; 12/16 browser/API tests passed before owner-requested closure. Four preference/search flows need retesting after fixes; PostgreSQL is unconfigured; port 3000 is closed. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 V5 adoption: V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="26" customHeight="1">
@@ -16976,7 +17010,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R189ad101049e4bae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fa981a2a59a45ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17013,7 +17047,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Foundation implemented, Pending runtime gates. 81 permanent IDs; append history. Port 3000 closed on owner request. Category tabs mirror open tasks; status tabs canonical.</x:v>
+        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -24658,7 +24692,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recece073434e4a04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc946a6e83e84fa8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24695,7 +24729,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Foundation implemented, Pending runtime gates. 81 permanent IDs; append history. Port 3000 closed on owner request. Category tabs mirror open tasks; status tabs canonical.</x:v>
+        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -32246,7 +32280,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Foundation implemented, Pending runtime gates. 81 permanent IDs; append history. Port 3000 closed on owner request. Category tabs mirror open tasks; status tabs canonical.</x:v>
+        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -32713,10 +32747,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F16" s="44" t="str">
-        <x:v>Preparation and foundation implemented; docs/tracker/source mirror updated. Build passes; 12/16 browser/API tests passed before owner-requested closure. Four preference/search flows need retesting after fixes; PostgreSQL is unconfigured; port 3000 is closed.</x:v>
+        <x:v>V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.</x:v>
       </x:c>
       <x:c r="G16" s="44" t="str">
-        <x:v>Codex: stop before Step 2. Retest only when owner opens localhost; verify real PostgreSQL.</x:v>
+        <x:v>Owner: supply the next stage prompt or authorize deferred tests. Codex: follow V5 one stage at a time; do not automatically advance.</x:v>
       </x:c>
       <x:c r="H16" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -32725,19 +32759,20 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J16" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>Documentation/planning update only. No application tests run at owner request. Existing runtime test results remain in prior history. Workbook/source/mirror checks performed.</x:v>
       </x:c>
       <x:c r="K16" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding foundation commit 604c62e pushed. V5 adoption commit/push verified at finalization; final report provides hash.</x:v>
       </x:c>
       <x:c r="L16" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>Baseline live files compared with Git before synchronization; revised guide/source/docs/tracker synchronized only after divergence checks.</x:v>
       </x:c>
       <x:c r="M16" s="44" t="str">
         <x:v>2026-10-09: Preparation recorded. Pending real-app/DB tests and localhost verification. Preserve this ID for subsequent updates.
 2026-10-09: cd897da pushed. Six sheets rendered; 81 IDs verified; 79 original IDs preserved. Preparation mirror hashes pass. R01 remains Pending for real-app/DB tests and localhost verification.
 2026-10-09 owner update: Owner choices documented and tracker updated. Foundation remains unbuilt; no app, PostgreSQL configuration or verified localhost URLs. Runtime gates remain pending.
-2026-10-09 foundation: Preparation and foundation implemented; docs/tracker/source mirror updated. Build passes; 12/16 browser/API tests passed before owner-requested closure. Four preference/search flows need retesting after fixes; PostgreSQL is unconfigured; port 3000 is closed. Owner requested localhost closure; do not reopen automatically.</x:v>
+2026-10-09 foundation: Preparation and foundation implemented; docs/tracker/source mirror updated. Build passes; 12/16 browser/API tests passed before owner-requested closure. Four preference/search flows need retesting after fixes; PostgreSQL is unconfigured; port 3000 is closed. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 V5 adoption: V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="250" customHeight="1">
@@ -40185,7 +40220,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R193e42a6cff2492e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dcf99137e75432f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40222,7 +40257,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Foundation implemented, Pending runtime gates. 81 permanent IDs; append history. Port 3000 closed on owner request. Category tabs mirror open tasks; status tabs canonical.</x:v>
+        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -40307,7 +40342,7 @@
         <x:v>History</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="26" customHeight="1">
+    <x:row r="6" ht="250" customHeight="1">
       <x:c r="A6" s="46" t="str">
         <x:v>F08</x:v>
       </x:c>
@@ -40315,7 +40350,7 @@
         <x:v>Step 3 · Cards</x:v>
       </x:c>
       <x:c r="C6" s="44" t="str">
-        <x:v>4:3 cards, photo galleries, save heart, badges and type-specific facts</x:v>
+        <x:v>Realtor-style 3:2 listing cards, photo controls, bottom-right save heart, facts/address and Contact agent dialog trigger</x:v>
       </x:c>
       <x:c r="D6" s="44" t="str">
         <x:v>Frontend</x:v>
@@ -40324,17 +40359,28 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="F6" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
+        <x:v>V5 Step 3 and revised BUILD-SPEC 4.3 replace the older 4:3 card plan. One reusable card across homepage/results/Saved. Not implemented; requires Step 2 Done.</x:v>
       </x:c>
       <x:c r="G6" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
+        <x:v>Codex: build revised card only under Step 3 authorization, after the real database step.</x:v>
       </x:c>
       <x:c r="H6" s="45"/>
-      <x:c r="I6" s="45"/>
-      <x:c r="J6" s="44"/>
-      <x:c r="K6" s="44"/>
-      <x:c r="L6" s="44"/>
-      <x:c r="M6" s="44"/>
+      <x:c r="I6" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J6" s="44" t="str">
+        <x:v>Documentation/planning update only. No application tests run at owner request. Existing runtime test results remain in prior history. Workbook/source/mirror checks performed.</x:v>
+      </x:c>
+      <x:c r="K6" s="44" t="str">
+        <x:v>Preceding foundation commit 604c62e pushed. V5 adoption commit/push verified at finalization; final report provides hash.</x:v>
+      </x:c>
+      <x:c r="L6" s="44" t="str">
+        <x:v>Baseline live files compared with Git before synchronization; revised guide/source/docs/tracker synchronized only after divergence checks.</x:v>
+      </x:c>
+      <x:c r="M6" s="44" t="str">
+        <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
+2026-10-09 V5 adoption: V5 Step 3 and revised BUILD-SPEC 4.3 replace the older 4:3 card plan. One reusable card across homepage/results/Saved. Not implemented; requires Step 2 Done.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="26" customHeight="1">
       <x:c r="A7" s="46" t="str">
@@ -40684,7 +40730,7 @@
       <x:c r="L18" s="44"/>
       <x:c r="M18" s="44"/>
     </x:row>
-    <x:row r="19" ht="26" customHeight="1">
+    <x:row r="19" ht="250" customHeight="1">
       <x:c r="A19" s="46" t="str">
         <x:v>F21</x:v>
       </x:c>
@@ -40692,7 +40738,7 @@
         <x:v>Step 6 · Contact</x:v>
       </x:c>
       <x:c r="C19" s="44" t="str">
-        <x:v>Desktop sticky enquiry box and phone sticky action bar</x:v>
+        <x:v>Shared agent enquiry form, card Contact agent dialog, desktop sticky box and phone contact bar</x:v>
       </x:c>
       <x:c r="D19" s="44" t="str">
         <x:v>Frontend</x:v>
@@ -40701,17 +40747,28 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="F19" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
+        <x:v>V5 Step 6 wires the card dialog and property form through one component/action. No implementation started; destinations still unresolved.</x:v>
       </x:c>
       <x:c r="G19" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
+        <x:v>Owner: provide routing/contacts. Codex: implement only under Step 6 authorization.</x:v>
       </x:c>
       <x:c r="H19" s="45"/>
-      <x:c r="I19" s="45"/>
-      <x:c r="J19" s="44"/>
-      <x:c r="K19" s="44"/>
-      <x:c r="L19" s="44"/>
-      <x:c r="M19" s="44"/>
+      <x:c r="I19" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J19" s="44" t="str">
+        <x:v>Documentation/planning update only. No application tests run at owner request. Existing runtime test results remain in prior history. Workbook/source/mirror checks performed.</x:v>
+      </x:c>
+      <x:c r="K19" s="44" t="str">
+        <x:v>Preceding foundation commit 604c62e pushed. V5 adoption commit/push verified at finalization; final report provides hash.</x:v>
+      </x:c>
+      <x:c r="L19" s="44" t="str">
+        <x:v>Baseline live files compared with Git before synchronization; revised guide/source/docs/tracker synchronized only after divergence checks.</x:v>
+      </x:c>
+      <x:c r="M19" s="44" t="str">
+        <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
+2026-10-09 V5 adoption: V5 Step 6 wires the card dialog and property form through one component/action. No implementation started; destinations still unresolved.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="26" customHeight="1">
       <x:c r="A20" s="46" t="str">
@@ -40800,7 +40857,7 @@
       <x:c r="L22" s="44"/>
       <x:c r="M22" s="44"/>
     </x:row>
-    <x:row r="23" ht="26" customHeight="1">
+    <x:row r="23" ht="250" customHeight="1">
       <x:c r="A23" s="46" t="str">
         <x:v>F25</x:v>
       </x:c>
@@ -40808,7 +40865,7 @@
         <x:v>Step 7 · Home</x:v>
       </x:c>
       <x:c r="C23" s="44" t="str">
-        <x:v>Featured homes, regions with accurate listing counts</x:v>
+        <x:v>Homes for you carousel directly below search; regions with real listing counts</x:v>
       </x:c>
       <x:c r="D23" s="44" t="str">
         <x:v>Frontend</x:v>
@@ -40817,17 +40874,28 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="F23" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
+        <x:v>V5 Step 7 uses Step 3 cards: five tabs, arrows, See all, 3/2/1.1 visible cards, swipe/scroll-snap, featured first then newest, up to 12 per tab. Not implemented.</x:v>
       </x:c>
       <x:c r="G23" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
+        <x:v>Codex: implement approved home-page.html only under Step 7 authorization.</x:v>
       </x:c>
       <x:c r="H23" s="45"/>
-      <x:c r="I23" s="45"/>
-      <x:c r="J23" s="44"/>
-      <x:c r="K23" s="44"/>
-      <x:c r="L23" s="44"/>
-      <x:c r="M23" s="44"/>
+      <x:c r="I23" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J23" s="44" t="str">
+        <x:v>Documentation/planning update only. No application tests run at owner request. Existing runtime test results remain in prior history. Workbook/source/mirror checks performed.</x:v>
+      </x:c>
+      <x:c r="K23" s="44" t="str">
+        <x:v>Preceding foundation commit 604c62e pushed. V5 adoption commit/push verified at finalization; final report provides hash.</x:v>
+      </x:c>
+      <x:c r="L23" s="44" t="str">
+        <x:v>Baseline live files compared with Git before synchronization; revised guide/source/docs/tracker synchronized only after divergence checks.</x:v>
+      </x:c>
+      <x:c r="M23" s="44" t="str">
+        <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
+2026-10-09 V5 adoption: V5 Step 7 uses Step 3 cards: five tabs, arrows, See all, 3/2/1.1 visible cards, swipe/scroll-snap, featured first then newest, up to 12 per tab. Not implemented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="26" customHeight="1">
       <x:c r="A24" s="46" t="str">
@@ -48654,7 +48722,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e60dd5e858d4191"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd923c45a72a64d84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(db): add PostgreSQL schema migrations and fictional seed
</commit_message>
<xml_diff>
--- a/Mstar-Property-Task-Tracker.xlsx
+++ b/Mstar-Property-Task-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="1" r:id="R4a40b80151914e17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="2" r:id="R649c040592ee4b5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" r:id="Ra0cb1649582144db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Done" sheetId="4" r:id="R351d6b6b298b4723"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="5" r:id="R4e7644ae36de49bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not started" sheetId="6" r:id="Rd670fa657f854d60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="1" r:id="R15871fd3ebf54e99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="2" r:id="R1362a8b864124b5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" r:id="Rc2942399b44044d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Done" sheetId="4" r:id="Rcd0af78f991b47a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="5" r:id="R4056639bf4294f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not started" sheetId="6" r:id="Rf51eb27c7f0246b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -356,7 +356,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="MstarFrontendTasks" displayName="MstarFrontendTasks" ref="A5:M43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="MstarFrontendTasks" displayName="MstarFrontendTasks" ref="A5:M43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -377,7 +377,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="MstarBackendTasks" displayName="MstarBackendTasks" ref="A5:M40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="MstarBackendTasks" displayName="MstarBackendTasks" ref="A5:M35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -398,7 +398,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="MstarEmailsTasks" displayName="MstarEmailsTasks" ref="A5:M13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="MstarEmailsTasks" displayName="MstarEmailsTasks" ref="A5:M13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -419,7 +419,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="MstarPendingTasks" displayName="MstarPendingTasks" ref="A5:M22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="MstarDoneTasks" displayName="MstarDoneTasks" ref="A5:M10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -440,7 +440,28 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="MstarNotstartedTasks" displayName="MstarNotstartedTasks" ref="A5:M69" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="MstarPendingTasks" displayName="MstarPendingTasks" ref="A5:M21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="ID"/>
+    <x:tableColumn id="2" name="Area"/>
+    <x:tableColumn id="3" name="Task"/>
+    <x:tableColumn id="4" name="Side"/>
+    <x:tableColumn id="5" name="Status"/>
+    <x:tableColumn id="6" name="Why / waiting for / evidence"/>
+    <x:tableColumn id="7" name="Next step (who)"/>
+    <x:tableColumn id="8" name="Created date"/>
+    <x:tableColumn id="9" name="Updated date"/>
+    <x:tableColumn id="10" name="Test results"/>
+    <x:tableColumn id="11" name="Git / push"/>
+    <x:tableColumn id="12" name="Live synchronization"/>
+    <x:tableColumn id="13" name="History"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="MstarNotstartedTasks" displayName="MstarNotstartedTasks" ref="A5:M65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -683,7 +704,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
+        <x:v>2026-10-09: Step 2 verified PostgreSQL schema/seed. 81 permanent IDs: 5 Done, 16 Pending, 60 Not started. Preserve append-only history. Test servers stop afterward.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -705,14 +726,14 @@
       </x:c>
       <x:c r="D3" s="18" t="n">
         <x:f>COUNTA('Done'!A6:A500)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F3" s="18" t="n">
         <x:f>COUNTA('Pending'!A6:A500)</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
         <x:v>Not started</x:v>
@@ -724,7 +745,7 @@
       </x:c>
       <x:c r="G4" s="22" t="n">
         <x:f>COUNTA('Not started'!A6:A500)</x:f>
-        <x:v>64</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
@@ -768,7 +789,7 @@
         <x:v>History</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="250" customHeight="1">
+    <x:row r="6" ht="310" customHeight="1">
       <x:c r="A6" s="46" t="str">
         <x:v>F02</x:v>
       </x:c>
@@ -785,10 +806,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F6" s="44" t="str">
-        <x:v>Approved gold and all section 2 colour tokens implemented and checked in eight shell tests. Overall runtime gates remain pending.</x:v>
+        <x:v>Owner approves gold / blue / teal / coral accent: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G6" s="44" t="str">
-        <x:v>Codex: preserve approved colours; complete remaining runtime gates.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H6" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -797,18 +818,20 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J6" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K6" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L6" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M6" s="44" t="str">
         <x:v>Original planning evidence: BUILD-SPEC §12 #1: accent not finalized
 2026-10-09 owner update: Owner selected approved wireframe colours: default gold #f2a91a and associated V3 tokens. Choice recorded; implementation/runtime completion gates remain pending.
-2026-10-09 foundation: Approved gold and all section 2 colour tokens implemented and checked in eight shell tests. Overall runtime gates remain pending. Owner requested localhost closure; do not reopen automatically.</x:v>
+2026-10-09 foundation: Approved gold and all section 2 colour tokens implemented and checked in eight shell tests. Overall runtime gates remain pending. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Approved gold and all section 2 colour tokens implemented and checked in eight shell tests. Overall runtime gates remain pending. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Owner approves gold / blue / teal / coral accent: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="250" customHeight="1">
@@ -912,7 +935,7 @@
       <x:c r="L9" s="44"/>
       <x:c r="M9" s="44"/>
     </x:row>
-    <x:row r="10" ht="250" customHeight="1">
+    <x:row r="10" ht="310" customHeight="1">
       <x:c r="A10" s="46" t="str">
         <x:v>F01</x:v>
       </x:c>
@@ -929,10 +952,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F10" s="44" t="str">
-        <x:v>Exact tokens, self-hosted fonts and reusable buttons/inputs/chips/tabs/dialogs/skeletons/search fields implemented. Final browser retests and real PostgreSQL completion gate remain pending.</x:v>
+        <x:v>Approved V3 CSS tokens, Prompt/Noto Sans Thai fonts, shared UI primitives: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G10" s="44" t="str">
-        <x:v>Codex: retest compiled final fixes when owner opens localhost; verify database gate.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H10" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -941,20 +964,22 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J10" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K10" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L10" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M10" s="44" t="str">
         <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
-2026-10-09 foundation: Exact tokens, self-hosted fonts and reusable buttons/inputs/chips/tabs/dialogs/skeletons/search fields implemented. Final browser retests and real PostgreSQL completion gate remain pending. Owner requested localhost closure; do not reopen automatically.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="250" customHeight="1">
+2026-10-09 foundation: Exact tokens, self-hosted fonts and reusable buttons/inputs/chips/tabs/dialogs/skeletons/search fields implemented. Final browser retests and real PostgreSQL completion gate remain pending. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Exact tokens, self-hosted fonts and reusable buttons/inputs/chips/tabs/dialogs/skeletons/search fields implemented. Final browser retests and real PostgreSQL completion gate remain pending. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Approved V3 CSS tokens, Prompt/Noto Sans Thai fonts, shared UI primitives: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="310" customHeight="1">
       <x:c r="A11" s="46" t="str">
         <x:v>F04</x:v>
       </x:c>
@@ -971,10 +996,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F11" s="44" t="str">
-        <x:v>Sticky 64px header, five desktop links, language/currency selector, Saved and rectangular Sign in implemented. All eight shell tests passed. Preference save fix needs retesting.</x:v>
+        <x:v>Sticky desktop header with one-line navigation and rectangular Sign in: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G11" s="44" t="str">
-        <x:v>Codex: retest preference flow when owner explicitly opens localhost.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H11" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -983,20 +1008,22 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J11" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K11" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L11" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M11" s="44" t="str">
         <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
-2026-10-09 foundation: Sticky 64px header, five desktop links, language/currency selector, Saved and rectangular Sign in implemented. All eight shell tests passed. Preference save fix needs retesting. Owner requested localhost closure; do not reopen automatically.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="250" customHeight="1">
+2026-10-09 foundation: Sticky 64px header, five desktop links, language/currency selector, Saved and rectangular Sign in implemented. All eight shell tests passed. Preference save fix needs retesting. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Sticky 64px header, five desktop links, language/currency selector, Saved and rectangular Sign in implemented. All eight shell tests passed. Preference save fix needs retesting. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Sticky desktop header with one-line navigation and rectangular Sign in: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="310" customHeight="1">
       <x:c r="A12" s="46" t="str">
         <x:v>F05</x:v>
       </x:c>
@@ -1013,10 +1040,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F12" s="44" t="str">
-        <x:v>Responsive phone header and five safe-area bottom tabs implemented. 390px Thai/English shell tests passed. Final phone search containment change needs retesting.</x:v>
+        <x:v>Phone header, bottom tabs and responsive breakpoints: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G12" s="44" t="str">
-        <x:v>Codex: retest final phone search containment when localhost is opened.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H12" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -1025,20 +1052,22 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J12" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K12" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L12" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M12" s="44" t="str">
         <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
-2026-10-09 foundation: Responsive phone header and five safe-area bottom tabs implemented. 390px Thai/English shell tests passed. Final phone search containment change needs retesting. Owner requested localhost closure; do not reopen automatically.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="250" customHeight="1">
+2026-10-09 foundation: Responsive phone header and five safe-area bottom tabs implemented. 390px Thai/English shell tests passed. Final phone search containment change needs retesting. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Responsive phone header and five safe-area bottom tabs implemented. 390px Thai/English shell tests passed. Final phone search containment change needs retesting. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Phone header, bottom tabs and responsive breakpoints: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="310" customHeight="1">
       <x:c r="A13" s="46" t="str">
         <x:v>F06</x:v>
       </x:c>
@@ -1055,10 +1084,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F13" s="44" t="str">
-        <x:v>Approved soft-background footer with bilingual company/area/help links implemented. Actual LINE ID omitted until provided. Shell tests passed.</x:v>
+        <x:v>Light footer, company links, contact and PDPA link: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G13" s="44" t="str">
-        <x:v>Owner: supply contact details; Codex: complete runtime gates.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H13" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -1067,20 +1096,22 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J13" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K13" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L13" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M13" s="44" t="str">
         <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
-2026-10-09 foundation: Approved soft-background footer with bilingual company/area/help links implemented. Actual LINE ID omitted until provided. Shell tests passed. Owner requested localhost closure; do not reopen automatically.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="250" customHeight="1">
+2026-10-09 foundation: Approved soft-background footer with bilingual company/area/help links implemented. Actual LINE ID omitted until provided. Shell tests passed. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Approved soft-background footer with bilingual company/area/help links implemented. Actual LINE ID omitted until provided. Shell tests passed. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Light footer, company links, contact and PDPA link: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="310" customHeight="1">
       <x:c r="A14" s="46" t="str">
         <x:v>F07</x:v>
       </x:c>
@@ -1097,10 +1128,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F14" s="44" t="str">
-        <x:v>Thai/English routes, Accept-Language and explicit preference cookies implemented. Redirect checks passed. Four browser preference/search flows failed before closure; Host-based origin fix compiles but remains untested in browser.</x:v>
+        <x:v>Thai/English routes, language switch and localized formatting: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G14" s="44" t="str">
-        <x:v>Codex: rerun preference persistence and search tests when owner opens localhost.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H14" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -1109,17 +1140,19 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J14" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K14" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L14" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M14" s="44" t="str">
         <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
-2026-10-09 foundation: Thai/English routes, Accept-Language and explicit preference cookies implemented. Redirect checks passed. Four browser preference/search flows failed before closure; Host-based origin fix compiles but remains untested in browser. Owner requested localhost closure; do not reopen automatically.</x:v>
+2026-10-09 foundation: Thai/English routes, Accept-Language and explicit preference cookies implemented. Redirect checks passed. Four browser preference/search flows failed before closure; Host-based origin fix compiles but remains untested in browser. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Thai/English routes, Accept-Language and explicit preference cookies implemented. Redirect checks passed. Four browser preference/search flows failed before closure; Host-based origin fix compiles but remains untested in browser. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Thai/English routes, language switch and localized formatting: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="250" customHeight="1">
@@ -8874,7 +8907,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R009d4f61af814f26"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13bbbb35cb3e4ec6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8911,7 +8944,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
+        <x:v>2026-10-09: Step 2 verified PostgreSQL schema/seed. 81 permanent IDs: 5 Done, 16 Pending, 60 Not started. Preserve append-only history. Test servers stop afterward.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -8933,14 +8966,14 @@
       </x:c>
       <x:c r="D3" s="18" t="n">
         <x:f>COUNTA('Done'!A6:A500)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F3" s="18" t="n">
         <x:f>COUNTA('Pending'!A6:A500)</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
         <x:v>Not started</x:v>
@@ -8952,7 +8985,7 @@
       </x:c>
       <x:c r="G4" s="22" t="n">
         <x:f>COUNTA('Not started'!A6:A500)</x:f>
-        <x:v>64</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
@@ -8996,7 +9029,7 @@
         <x:v>History</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="200" customHeight="1">
+    <x:row r="6" ht="310" customHeight="1">
       <x:c r="A6" s="46" t="str">
         <x:v>B09</x:v>
       </x:c>
@@ -9004,7 +9037,7 @@
         <x:v>Decision · Map</x:v>
       </x:c>
       <x:c r="C6" s="44" t="str">
-        <x:v>Approve Google Maps Platform or Longdo Map</x:v>
+        <x:v>Select free open-source map library, tile/nearby provider and usage policy</x:v>
       </x:c>
       <x:c r="D6" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9013,27 +9046,30 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F6" s="44" t="str">
-        <x:v>Owner requests free open-source mapping for now. Specific library and tile/nearby provider remain undecided.</x:v>
+        <x:v>Owner/V5 require free open-source mapping. Concrete provider/library/policy remain unresolved; Step 2 makes no choice.</x:v>
       </x:c>
       <x:c r="G6" s="44" t="str">
-        <x:v>Codex: evaluate free open-source mapping before map step; confirm provider and usage policy.</x:v>
-      </x:c>
-      <x:c r="H6" s="45"/>
+        <x:v>Codex: present free options and wait for owner choice under Step 4 authorization.</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="I6" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J6" s="44" t="str">
-        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K6" s="44" t="str">
-        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L6" s="44" t="str">
-        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M6" s="44" t="str">
         <x:v>Original planning evidence: BUILD-SPEC §12 #8: map provider not selected
-2026-10-09 owner update: Owner requests free open-source mapping for now. Specific library and tile/nearby provider remain undecided.</x:v>
+2026-10-09 owner update: Owner requests free open-source mapping for now. Specific library and tile/nearby provider remain undecided.
+2026-10-09 Step 2: Owner/V5 require free open-source mapping. Concrete provider/library/policy remain unresolved; Step 2 makes no choice. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="26" customHeight="1">
@@ -9217,7 +9253,7 @@
 2026-10-09 owner update: Owner selected both public and contact-gated pricing, chosen by admin per listing/product or project. Choice recorded; implementation pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="250" customHeight="1">
+    <x:row r="12" ht="310" customHeight="1">
       <x:c r="A12" s="46" t="str">
         <x:v>R01</x:v>
       </x:c>
@@ -9234,10 +9270,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F12" s="44" t="str">
-        <x:v>V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.</x:v>
+        <x:v>Step 2 schema/seed/runtime tests pass. Preparation closeout remains separate: V5 Step 0 tracker-update utility is not in the project and original local prototype rendering is browser-policy blocked. No duplicate IDs or source changes. Servers stop under latest request.</x:v>
       </x:c>
       <x:c r="G12" s="44" t="str">
-        <x:v>Owner: supply the next stage prompt or authorize deferred tests. Codex: follow V5 one stage at a time; do not automatically advance.</x:v>
+        <x:v>Codex: close the separate Step 0 utility/reference-review requirements only when authorized; stop before Step 3.</x:v>
       </x:c>
       <x:c r="H12" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -9246,31 +9282,32 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J12" s="44" t="str">
-        <x:v>Documentation/planning update only. No application tests run at owner request. Existing runtime test results remain in prior history. Workbook/source/mirror checks performed.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K12" s="44" t="str">
-        <x:v>Preceding foundation commit 604c62e pushed. V5 adoption commit/push verified at finalization; final report provides hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L12" s="44" t="str">
-        <x:v>Baseline live files compared with Git before synchronization; revised guide/source/docs/tracker synchronized only after divergence checks.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M12" s="44" t="str">
         <x:v>2026-10-09: Preparation recorded. Pending real-app/DB tests and localhost verification. Preserve this ID for subsequent updates.
 2026-10-09: cd897da pushed. Six sheets rendered; 81 IDs verified; 79 original IDs preserved. Preparation mirror hashes pass. R01 remains Pending for real-app/DB tests and localhost verification.
 2026-10-09 owner update: Owner choices documented and tracker updated. Foundation remains unbuilt; no app, PostgreSQL configuration or verified localhost URLs. Runtime gates remain pending.
 2026-10-09 foundation: Preparation and foundation implemented; docs/tracker/source mirror updated. Build passes; 12/16 browser/API tests passed before owner-requested closure. Four preference/search flows need retesting after fixes; PostgreSQL is unconfigured; port 3000 is closed. Owner requested localhost closure; do not reopen automatically.
-2026-10-09 V5 adoption: V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.</x:v>
+2026-10-09 V5 adoption: V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.
+2026-10-09 Step 2: Step 2 schema/seed/runtime tests pass. Preparation closeout remains separate: V5 Step 0 tracker-update utility is not in the project and original local prototype rendering is browser-policy blocked. No duplicate IDs or source changes. Servers stop under latest request. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="26" customHeight="1">
       <x:c r="A13" s="46" t="str">
-        <x:v>B01</x:v>
+        <x:v>B05</x:v>
       </x:c>
       <x:c r="B13" s="44" t="str">
-        <x:v>Step 2 · Database</x:v>
+        <x:v>Step 2 · Filters</x:v>
       </x:c>
       <x:c r="C13" s="44" t="str">
-        <x:v>PostgreSQL/Drizzle schema for listings, projects, agents and users</x:v>
+        <x:v>Configurable filter-definition/option tables with safe allowed query fields</x:v>
       </x:c>
       <x:c r="D13" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9293,13 +9330,13 @@
     </x:row>
     <x:row r="14" ht="26" customHeight="1">
       <x:c r="A14" s="46" t="str">
-        <x:v>B02</x:v>
+        <x:v>B06</x:v>
       </x:c>
       <x:c r="B14" s="44" t="str">
-        <x:v>Step 2 · Database</x:v>
+        <x:v>Step 3 · Search</x:v>
       </x:c>
       <x:c r="C14" s="44" t="str">
-        <x:v>Migrations, foreign keys, constraints and rollback procedure</x:v>
+        <x:v>Typed validated listing/search data access and pagination</x:v>
       </x:c>
       <x:c r="D14" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9322,13 +9359,13 @@
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
       <x:c r="A15" s="46" t="str">
-        <x:v>B03</x:v>
+        <x:v>B07</x:v>
       </x:c>
       <x:c r="B15" s="44" t="str">
-        <x:v>Step 2 · Demo</x:v>
+        <x:v>Step 3 · Search</x:v>
       </x:c>
       <x:c r="C15" s="44" t="str">
-        <x:v>Clearly fictional seed listings, projects and agents</x:v>
+        <x:v>Filter parsing, result counts, sort and histogram queries</x:v>
       </x:c>
       <x:c r="D15" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9351,13 +9388,13 @@
     </x:row>
     <x:row r="16" ht="26" customHeight="1">
       <x:c r="A16" s="46" t="str">
-        <x:v>B04</x:v>
+        <x:v>B08</x:v>
       </x:c>
       <x:c r="B16" s="44" t="str">
-        <x:v>Step 2 · Search</x:v>
+        <x:v>Step 4 · Map</x:v>
       </x:c>
       <x:c r="C16" s="44" t="str">
-        <x:v>Indexes for status, intent, type, price, location and title</x:v>
+        <x:v>Geospatial index, bounding-box search and hidden-pin privacy</x:v>
       </x:c>
       <x:c r="D16" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9380,13 +9417,13 @@
     </x:row>
     <x:row r="17" ht="26" customHeight="1">
       <x:c r="A17" s="46" t="str">
-        <x:v>B05</x:v>
+        <x:v>B10</x:v>
       </x:c>
       <x:c r="B17" s="44" t="str">
-        <x:v>Step 2 · Filters</x:v>
+        <x:v>Step 4 · Nearby</x:v>
       </x:c>
       <x:c r="C17" s="44" t="str">
-        <x:v>Configurable filter-definition/option tables with safe allowed query fields</x:v>
+        <x:v>Provider-backed nearby data ingest and 90-day refresh</x:v>
       </x:c>
       <x:c r="D17" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9409,13 +9446,13 @@
     </x:row>
     <x:row r="18" ht="26" customHeight="1">
       <x:c r="A18" s="46" t="str">
-        <x:v>B06</x:v>
+        <x:v>B11</x:v>
       </x:c>
       <x:c r="B18" s="44" t="str">
-        <x:v>Step 3 · Search</x:v>
+        <x:v>Step 5 · Media</x:v>
       </x:c>
       <x:c r="C18" s="44" t="str">
-        <x:v>Typed validated listing/search data access and pagination</x:v>
+        <x:v>Photo/floorplan/video metadata and safe image upload pipeline</x:v>
       </x:c>
       <x:c r="D18" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9438,13 +9475,13 @@
     </x:row>
     <x:row r="19" ht="26" customHeight="1">
       <x:c r="A19" s="46" t="str">
-        <x:v>B07</x:v>
+        <x:v>B12</x:v>
       </x:c>
       <x:c r="B19" s="44" t="str">
-        <x:v>Step 3 · Search</x:v>
+        <x:v>Step 5 · Similar</x:v>
       </x:c>
       <x:c r="C19" s="44" t="str">
-        <x:v>Filter parsing, result counts, sort and histogram queries</x:v>
+        <x:v>Same-location/type/intent matching with ±25% price fallback</x:v>
       </x:c>
       <x:c r="D19" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9467,13 +9504,13 @@
     </x:row>
     <x:row r="20" ht="26" customHeight="1">
       <x:c r="A20" s="46" t="str">
-        <x:v>B08</x:v>
+        <x:v>B13</x:v>
       </x:c>
       <x:c r="B20" s="44" t="str">
-        <x:v>Step 4 · Map</x:v>
+        <x:v>Step 5 · Metrics</x:v>
       </x:c>
       <x:c r="C20" s="44" t="str">
-        <x:v>Geospatial index, bounding-box search and hidden-pin privacy</x:v>
+        <x:v>Comparable pricing/yield gated by verified sample size</x:v>
       </x:c>
       <x:c r="D20" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9496,13 +9533,13 @@
     </x:row>
     <x:row r="21" ht="26" customHeight="1">
       <x:c r="A21" s="46" t="str">
-        <x:v>B10</x:v>
+        <x:v>B14</x:v>
       </x:c>
       <x:c r="B21" s="44" t="str">
-        <x:v>Step 4 · Nearby</x:v>
+        <x:v>Step 6 · Leads</x:v>
       </x:c>
       <x:c r="C21" s="44" t="str">
-        <x:v>Provider-backed nearby data ingest and 90-day refresh</x:v>
+        <x:v>Enquiry API validation and DB-first persist-before-notify flow</x:v>
       </x:c>
       <x:c r="D21" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9525,13 +9562,13 @@
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
       <x:c r="A22" s="46" t="str">
-        <x:v>B11</x:v>
+        <x:v>B15</x:v>
       </x:c>
       <x:c r="B22" s="44" t="str">
-        <x:v>Step 5 · Media</x:v>
+        <x:v>Step 6 · Leads</x:v>
       </x:c>
       <x:c r="C22" s="44" t="str">
-        <x:v>Photo/floorplan/video metadata and safe image upload pipeline</x:v>
+        <x:v>PDPA consent version, UTM/source, language and audit metadata</x:v>
       </x:c>
       <x:c r="D22" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9554,13 +9591,13 @@
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
       <x:c r="A23" s="46" t="str">
-        <x:v>B12</x:v>
+        <x:v>B16</x:v>
       </x:c>
       <x:c r="B23" s="44" t="str">
-        <x:v>Step 5 · Similar</x:v>
+        <x:v>Step 6 · Security</x:v>
       </x:c>
       <x:c r="C23" s="44" t="str">
-        <x:v>Same-location/type/intent matching with ±25% price fallback</x:v>
+        <x:v>Rate limits, honeypot and duplicate submission protection</x:v>
       </x:c>
       <x:c r="D23" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9583,13 +9620,13 @@
     </x:row>
     <x:row r="24" ht="26" customHeight="1">
       <x:c r="A24" s="46" t="str">
-        <x:v>B13</x:v>
+        <x:v>B19</x:v>
       </x:c>
       <x:c r="B24" s="44" t="str">
-        <x:v>Step 5 · Metrics</x:v>
+        <x:v>Step 6 · Chat</x:v>
       </x:c>
       <x:c r="C24" s="44" t="str">
-        <x:v>Comparable pricing/yield gated by verified sample size</x:v>
+        <x:v>Validated LINE/WhatsApp URLs and click event tracking</x:v>
       </x:c>
       <x:c r="D24" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9612,13 +9649,13 @@
     </x:row>
     <x:row r="25" ht="26" customHeight="1">
       <x:c r="A25" s="46" t="str">
-        <x:v>B14</x:v>
+        <x:v>B20</x:v>
       </x:c>
       <x:c r="B25" s="44" t="str">
-        <x:v>Step 6 · Leads</x:v>
+        <x:v>Step 8 · Projects</x:v>
       </x:c>
       <x:c r="C25" s="44" t="str">
-        <x:v>Enquiry API validation and DB-first persist-before-notify flow</x:v>
+        <x:v>Project/unit/plot status logic and validation</x:v>
       </x:c>
       <x:c r="D25" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9641,13 +9678,13 @@
     </x:row>
     <x:row r="26" ht="26" customHeight="1">
       <x:c r="A26" s="46" t="str">
-        <x:v>B15</x:v>
+        <x:v>B21</x:v>
       </x:c>
       <x:c r="B26" s="44" t="str">
-        <x:v>Step 6 · Leads</x:v>
+        <x:v>Step 8 · Booking</x:v>
       </x:c>
       <x:c r="C26" s="44" t="str">
-        <x:v>PDPA consent version, UTM/source, language and audit metadata</x:v>
+        <x:v>Site-visit availability and enquiry persistence, double-book protection</x:v>
       </x:c>
       <x:c r="D26" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9670,13 +9707,13 @@
     </x:row>
     <x:row r="27" ht="26" customHeight="1">
       <x:c r="A27" s="46" t="str">
-        <x:v>B16</x:v>
+        <x:v>B22</x:v>
       </x:c>
       <x:c r="B27" s="44" t="str">
-        <x:v>Step 6 · Security</x:v>
+        <x:v>Step 9 · Saved</x:v>
       </x:c>
       <x:c r="C27" s="44" t="str">
-        <x:v>Rate limits, honeypot and duplicate submission protection</x:v>
+        <x:v>Saved listings/searches persistence, new-match calculations</x:v>
       </x:c>
       <x:c r="D27" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9699,13 +9736,13 @@
     </x:row>
     <x:row r="28" ht="26" customHeight="1">
       <x:c r="A28" s="46" t="str">
-        <x:v>B19</x:v>
+        <x:v>B24</x:v>
       </x:c>
       <x:c r="B28" s="44" t="str">
-        <x:v>Step 6 · Chat</x:v>
+        <x:v>Step 10B · Auth</x:v>
       </x:c>
       <x:c r="C28" s="44" t="str">
-        <x:v>Validated LINE/WhatsApp URLs and click event tracking</x:v>
+        <x:v>Secure sessions, approved sign-in integrations and auth tests</x:v>
       </x:c>
       <x:c r="D28" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9728,13 +9765,13 @@
     </x:row>
     <x:row r="29" ht="26" customHeight="1">
       <x:c r="A29" s="46" t="str">
-        <x:v>B20</x:v>
+        <x:v>B25</x:v>
       </x:c>
       <x:c r="B29" s="44" t="str">
-        <x:v>Step 8 · Projects</x:v>
+        <x:v>Step 10B · Auth</x:v>
       </x:c>
       <x:c r="C29" s="44" t="str">
-        <x:v>Project/unit/plot status logic and validation</x:v>
+        <x:v>Account/localStorage saved-item merge and privacy isolation</x:v>
       </x:c>
       <x:c r="D29" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9757,13 +9794,13 @@
     </x:row>
     <x:row r="30" ht="26" customHeight="1">
       <x:c r="A30" s="46" t="str">
-        <x:v>B21</x:v>
+        <x:v>B26</x:v>
       </x:c>
       <x:c r="B30" s="44" t="str">
-        <x:v>Step 8 · Booking</x:v>
+        <x:v>Step 11B · Admin</x:v>
       </x:c>
       <x:c r="C30" s="44" t="str">
-        <x:v>Site-visit availability and enquiry persistence, double-book protection</x:v>
+        <x:v>Role-scoped CRUD for listings, images, projects, agents, filter config</x:v>
       </x:c>
       <x:c r="D30" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9786,13 +9823,13 @@
     </x:row>
     <x:row r="31" ht="26" customHeight="1">
       <x:c r="A31" s="46" t="str">
-        <x:v>B22</x:v>
+        <x:v>B27</x:v>
       </x:c>
       <x:c r="B31" s="44" t="str">
-        <x:v>Step 9 · Saved</x:v>
+        <x:v>Step 11B · Admin</x:v>
       </x:c>
       <x:c r="C31" s="44" t="str">
-        <x:v>Saved listings/searches persistence, new-match calculations</x:v>
+        <x:v>Admin user management, audit log and sensitive action authorization</x:v>
       </x:c>
       <x:c r="D31" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9815,13 +9852,13 @@
     </x:row>
     <x:row r="32" ht="26" customHeight="1">
       <x:c r="A32" s="46" t="str">
-        <x:v>B24</x:v>
+        <x:v>B30</x:v>
       </x:c>
       <x:c r="B32" s="44" t="str">
-        <x:v>Step 10B · Auth</x:v>
+        <x:v>Step 12 · Deploy</x:v>
       </x:c>
       <x:c r="C32" s="44" t="str">
-        <x:v>Secure sessions, approved sign-in integrations and auth tests</x:v>
+        <x:v>Single VPS deployment, TLS, backups and migration runbook</x:v>
       </x:c>
       <x:c r="D32" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9844,13 +9881,13 @@
     </x:row>
     <x:row r="33" ht="26" customHeight="1">
       <x:c r="A33" s="46" t="str">
-        <x:v>B25</x:v>
+        <x:v>B31</x:v>
       </x:c>
       <x:c r="B33" s="44" t="str">
-        <x:v>Step 10B · Auth</x:v>
+        <x:v>Step 12 · Quality</x:v>
       </x:c>
       <x:c r="C33" s="44" t="str">
-        <x:v>Account/localStorage saved-item merge and privacy isolation</x:v>
+        <x:v>Real PostgreSQL integration/Playwright tests and EXPLAIN ANALYZE</x:v>
       </x:c>
       <x:c r="D33" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9873,13 +9910,13 @@
     </x:row>
     <x:row r="34" ht="26" customHeight="1">
       <x:c r="A34" s="46" t="str">
-        <x:v>B26</x:v>
+        <x:v>B32</x:v>
       </x:c>
       <x:c r="B34" s="44" t="str">
-        <x:v>Step 11B · Admin</x:v>
+        <x:v>Step 12 · Security</x:v>
       </x:c>
       <x:c r="C34" s="44" t="str">
-        <x:v>Role-scoped CRUD for listings, images, projects, agents, filter config</x:v>
+        <x:v>Access control, PDPA, headers, secrets and rate-limit audit</x:v>
       </x:c>
       <x:c r="D34" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9902,13 +9939,13 @@
     </x:row>
     <x:row r="35" ht="26" customHeight="1">
       <x:c r="A35" s="46" t="str">
-        <x:v>B27</x:v>
+        <x:v>B33</x:v>
       </x:c>
       <x:c r="B35" s="44" t="str">
-        <x:v>Step 11B · Admin</x:v>
+        <x:v>Step 7 · Owners</x:v>
       </x:c>
       <x:c r="C35" s="44" t="str">
-        <x:v>Admin user management, audit log and sensitive action authorization</x:v>
+        <x:v>Home-value and service enquiry data handling</x:v>
       </x:c>
       <x:c r="D35" s="44" t="str">
         <x:v>Backend</x:v>
@@ -9930,27 +9967,13 @@
       <x:c r="M35" s="44"/>
     </x:row>
     <x:row r="36" ht="26" customHeight="1">
-      <x:c r="A36" s="46" t="str">
-        <x:v>B30</x:v>
-      </x:c>
-      <x:c r="B36" s="44" t="str">
-        <x:v>Step 12 · Deploy</x:v>
-      </x:c>
-      <x:c r="C36" s="44" t="str">
-        <x:v>Single VPS deployment, TLS, backups and migration runbook</x:v>
-      </x:c>
-      <x:c r="D36" s="44" t="str">
-        <x:v>Backend</x:v>
-      </x:c>
-      <x:c r="E36" s="44" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F36" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
-      </x:c>
-      <x:c r="G36" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
-      </x:c>
+      <x:c r="A36" s="46"/>
+      <x:c r="B36" s="44"/>
+      <x:c r="C36" s="44"/>
+      <x:c r="D36" s="44"/>
+      <x:c r="E36" s="44"/>
+      <x:c r="F36" s="44"/>
+      <x:c r="G36" s="44"/>
       <x:c r="H36" s="45"/>
       <x:c r="I36" s="45"/>
       <x:c r="J36" s="44"/>
@@ -9959,27 +9982,13 @@
       <x:c r="M36" s="44"/>
     </x:row>
     <x:row r="37" ht="26" customHeight="1">
-      <x:c r="A37" s="46" t="str">
-        <x:v>B31</x:v>
-      </x:c>
-      <x:c r="B37" s="44" t="str">
-        <x:v>Step 12 · Quality</x:v>
-      </x:c>
-      <x:c r="C37" s="44" t="str">
-        <x:v>Real PostgreSQL integration/Playwright tests and EXPLAIN ANALYZE</x:v>
-      </x:c>
-      <x:c r="D37" s="44" t="str">
-        <x:v>Backend</x:v>
-      </x:c>
-      <x:c r="E37" s="44" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F37" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
-      </x:c>
-      <x:c r="G37" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
-      </x:c>
+      <x:c r="A37" s="46"/>
+      <x:c r="B37" s="44"/>
+      <x:c r="C37" s="44"/>
+      <x:c r="D37" s="44"/>
+      <x:c r="E37" s="44"/>
+      <x:c r="F37" s="44"/>
+      <x:c r="G37" s="44"/>
       <x:c r="H37" s="45"/>
       <x:c r="I37" s="45"/>
       <x:c r="J37" s="44"/>
@@ -9988,27 +9997,13 @@
       <x:c r="M37" s="44"/>
     </x:row>
     <x:row r="38" ht="26" customHeight="1">
-      <x:c r="A38" s="46" t="str">
-        <x:v>B32</x:v>
-      </x:c>
-      <x:c r="B38" s="44" t="str">
-        <x:v>Step 12 · Security</x:v>
-      </x:c>
-      <x:c r="C38" s="44" t="str">
-        <x:v>Access control, PDPA, headers, secrets and rate-limit audit</x:v>
-      </x:c>
-      <x:c r="D38" s="44" t="str">
-        <x:v>Backend</x:v>
-      </x:c>
-      <x:c r="E38" s="44" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F38" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
-      </x:c>
-      <x:c r="G38" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
-      </x:c>
+      <x:c r="A38" s="46"/>
+      <x:c r="B38" s="44"/>
+      <x:c r="C38" s="44"/>
+      <x:c r="D38" s="44"/>
+      <x:c r="E38" s="44"/>
+      <x:c r="F38" s="44"/>
+      <x:c r="G38" s="44"/>
       <x:c r="H38" s="45"/>
       <x:c r="I38" s="45"/>
       <x:c r="J38" s="44"/>
@@ -10017,27 +10012,13 @@
       <x:c r="M38" s="44"/>
     </x:row>
     <x:row r="39" ht="200" customHeight="1">
-      <x:c r="A39" s="44" t="str">
-        <x:v>B33</x:v>
-      </x:c>
-      <x:c r="B39" s="44" t="str">
-        <x:v>Step 7 · Owners</x:v>
-      </x:c>
-      <x:c r="C39" s="44" t="str">
-        <x:v>Home-value and service enquiry data handling</x:v>
-      </x:c>
-      <x:c r="D39" s="44" t="str">
-        <x:v>Backend</x:v>
-      </x:c>
-      <x:c r="E39" s="44" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F39" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
-      </x:c>
-      <x:c r="G39" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
-      </x:c>
+      <x:c r="A39" s="44"/>
+      <x:c r="B39" s="44"/>
+      <x:c r="C39" s="44"/>
+      <x:c r="D39" s="44"/>
+      <x:c r="E39" s="44"/>
+      <x:c r="F39" s="44"/>
+      <x:c r="G39" s="44"/>
       <x:c r="H39" s="45"/>
       <x:c r="I39" s="45"/>
       <x:c r="J39" s="44"/>
@@ -10046,46 +10027,19 @@
       <x:c r="M39" s="44"/>
     </x:row>
     <x:row r="40" ht="250" customHeight="1">
-      <x:c r="A40" s="44" t="str">
-        <x:v>B34</x:v>
-      </x:c>
-      <x:c r="B40" s="44" t="str">
-        <x:v>Step 1 · Health</x:v>
-      </x:c>
-      <x:c r="C40" s="44" t="str">
-        <x:v>Basic /api/health endpoint with accurate application and database status</x:v>
-      </x:c>
-      <x:c r="D40" s="44" t="str">
-        <x:v>Backend</x:v>
-      </x:c>
-      <x:c r="E40" s="44" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="F40" s="44" t="str">
-        <x:v>Real health API implemented: HTTP 200 app ok, database not_configured, ready false before closure. Configured PostgreSQL is probed with Drizzle select 1; failure returns 503. No real database configuration exists.</x:v>
-      </x:c>
-      <x:c r="G40" s="44" t="str">
-        <x:v>Codex: verify against real PostgreSQL when configured and localhost opening is authorized.</x:v>
-      </x:c>
-      <x:c r="H40" s="45" t="d">
-        <x:v>2026-10-09T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="I40" s="45" t="d">
-        <x:v>2026-10-09T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="J40" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
-      </x:c>
-      <x:c r="K40" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
-      </x:c>
-      <x:c r="L40" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
-      </x:c>
-      <x:c r="M40" s="44" t="str">
-        <x:v>2026-10-09: Health API planned. No implementation in Step 0.
-2026-10-09 foundation: Real health API implemented: HTTP 200 app ok, database not_configured, ready false before closure. Configured PostgreSQL is probed with Drizzle select 1; failure returns 503. No real database configuration exists. Owner requested localhost closure; do not reopen automatically.</x:v>
-      </x:c>
+      <x:c r="A40" s="44"/>
+      <x:c r="B40" s="44"/>
+      <x:c r="C40" s="44"/>
+      <x:c r="D40" s="44"/>
+      <x:c r="E40" s="44"/>
+      <x:c r="F40" s="44"/>
+      <x:c r="G40" s="44"/>
+      <x:c r="H40" s="45"/>
+      <x:c r="I40" s="45"/>
+      <x:c r="J40" s="44"/>
+      <x:c r="K40" s="44"/>
+      <x:c r="L40" s="44"/>
+      <x:c r="M40" s="44"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="44"/>
@@ -17003,14 +16957,17 @@
       <x:formula>E6="Not started"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="E6:E40">
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="E36:E40">
+      <x:formula1>"Done,Pending,Not started"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E6:E35">
       <x:formula1>"Done,Pending,Not started"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fa981a2a59a45ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf97900a44a464015"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17047,7 +17004,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
+        <x:v>2026-10-09: Step 2 verified PostgreSQL schema/seed. 81 permanent IDs: 5 Done, 16 Pending, 60 Not started. Preserve append-only history. Test servers stop afterward.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -17069,14 +17026,14 @@
       </x:c>
       <x:c r="D3" s="18" t="n">
         <x:f>COUNTA('Done'!A6:A500)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F3" s="18" t="n">
         <x:f>COUNTA('Pending'!A6:A500)</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
         <x:v>Not started</x:v>
@@ -17088,7 +17045,7 @@
       </x:c>
       <x:c r="G4" s="22" t="n">
         <x:f>COUNTA('Not started'!A6:A500)</x:f>
-        <x:v>64</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
@@ -24692,7 +24649,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc946a6e83e84fa8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a3d0235b3e94810"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24729,7 +24686,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
+        <x:v>2026-10-09: Step 2 verified PostgreSQL schema/seed. 81 permanent IDs: 5 Done, 16 Pending, 60 Not started. Preserve append-only history. Test servers stop afterward.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -24751,14 +24708,14 @@
       </x:c>
       <x:c r="D3" s="18" t="n">
         <x:f>COUNTA('Done'!A6:A500)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F3" s="18" t="n">
         <x:f>COUNTA('Pending'!A6:A500)</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
         <x:v>Not started</x:v>
@@ -24770,7 +24727,7 @@
       </x:c>
       <x:c r="G4" s="22" t="n">
         <x:f>COUNTA('Not started'!A6:A500)</x:f>
-        <x:v>64</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
@@ -24814,80 +24771,216 @@
         <x:v>History</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="44"/>
-      <x:c r="B6" s="44"/>
-      <x:c r="C6" s="44"/>
-      <x:c r="D6" s="44"/>
-      <x:c r="E6" s="44"/>
-      <x:c r="F6" s="44"/>
-      <x:c r="G6" s="44"/>
-      <x:c r="H6" s="45"/>
-      <x:c r="I6" s="45"/>
-      <x:c r="J6" s="44"/>
-      <x:c r="K6" s="44"/>
-      <x:c r="L6" s="44"/>
-      <x:c r="M6" s="44"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="44"/>
-      <x:c r="B7" s="44"/>
-      <x:c r="C7" s="44"/>
-      <x:c r="D7" s="44"/>
-      <x:c r="E7" s="44"/>
-      <x:c r="F7" s="44"/>
-      <x:c r="G7" s="44"/>
-      <x:c r="H7" s="45"/>
-      <x:c r="I7" s="45"/>
-      <x:c r="J7" s="44"/>
-      <x:c r="K7" s="44"/>
-      <x:c r="L7" s="44"/>
-      <x:c r="M7" s="44"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="44"/>
-      <x:c r="B8" s="44"/>
-      <x:c r="C8" s="44"/>
-      <x:c r="D8" s="44"/>
-      <x:c r="E8" s="44"/>
-      <x:c r="F8" s="44"/>
-      <x:c r="G8" s="44"/>
-      <x:c r="H8" s="45"/>
-      <x:c r="I8" s="45"/>
-      <x:c r="J8" s="44"/>
-      <x:c r="K8" s="44"/>
-      <x:c r="L8" s="44"/>
-      <x:c r="M8" s="44"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="44"/>
-      <x:c r="B9" s="44"/>
-      <x:c r="C9" s="44"/>
-      <x:c r="D9" s="44"/>
-      <x:c r="E9" s="44"/>
-      <x:c r="F9" s="44"/>
-      <x:c r="G9" s="44"/>
-      <x:c r="H9" s="45"/>
-      <x:c r="I9" s="45"/>
-      <x:c r="J9" s="44"/>
-      <x:c r="K9" s="44"/>
-      <x:c r="L9" s="44"/>
-      <x:c r="M9" s="44"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="44"/>
-      <x:c r="B10" s="44"/>
-      <x:c r="C10" s="44"/>
-      <x:c r="D10" s="44"/>
-      <x:c r="E10" s="44"/>
-      <x:c r="F10" s="44"/>
-      <x:c r="G10" s="44"/>
-      <x:c r="H10" s="45"/>
-      <x:c r="I10" s="45"/>
-      <x:c r="J10" s="44"/>
-      <x:c r="K10" s="44"/>
-      <x:c r="L10" s="44"/>
-      <x:c r="M10" s="44"/>
+    <x:row r="6" ht="310" customHeight="1">
+      <x:c r="A6" s="44" t="str">
+        <x:v>B34</x:v>
+      </x:c>
+      <x:c r="B6" s="44" t="str">
+        <x:v>Step 1 · Health</x:v>
+      </x:c>
+      <x:c r="C6" s="44" t="str">
+        <x:v>Basic /api/health endpoint with accurate application and database status</x:v>
+      </x:c>
+      <x:c r="D6" s="44" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="E6" s="44" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F6" s="44" t="str">
+        <x:v>Real /api/health now probes the migrated public view rather than an empty database select 1. Actual 200/ready true, stopped-DB 503/unavailable/ready false and recovery to 200 verified.</x:v>
+      </x:c>
+      <x:c r="G6" s="44" t="str">
+        <x:v>Codex: retain truthful readiness and generic errors; start localhost only under owner/test authorization.</x:v>
+      </x:c>
+      <x:c r="H6" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I6" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J6" s="44" t="str">
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+      <x:c r="K6" s="44" t="str">
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
+      </x:c>
+      <x:c r="L6" s="44" t="str">
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
+      </x:c>
+      <x:c r="M6" s="44" t="str">
+        <x:v>2026-10-09: Health API planned. No implementation in Step 0.
+2026-10-09 foundation: Real health API implemented: HTTP 200 app ok, database not_configured, ready false before closure. Configured PostgreSQL is probed with Drizzle select 1; failure returns 503. No real database configuration exists. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Real /api/health now probes the migrated public view rather than an empty database select 1. Actual 200/ready true, stopped-DB 503/unavailable/ready false and recovery to 200 verified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="310" customHeight="1">
+      <x:c r="A7" s="44" t="str">
+        <x:v>B01</x:v>
+      </x:c>
+      <x:c r="B7" s="44" t="str">
+        <x:v>Step 2 · Database</x:v>
+      </x:c>
+      <x:c r="C7" s="44" t="str">
+        <x:v>PostgreSQL/Drizzle schema for listings, projects, agents and users</x:v>
+      </x:c>
+      <x:c r="D7" s="44" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="E7" s="44" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F7" s="44" t="str">
+        <x:v>18-table Drizzle schema implemented with bilingual fields, seven property types, sale/rent rules, explicit price visibility and separate non-superuser migration/read-only app roles. Isolated local development/test PostgreSQL configured; no shared service modified.</x:v>
+      </x:c>
+      <x:c r="G7" s="44" t="str">
+        <x:v>Codex: preserve schema/security contracts in later explicitly authorized stages.</x:v>
+      </x:c>
+      <x:c r="H7" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I7" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J7" s="44" t="str">
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+      <x:c r="K7" s="44" t="str">
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
+      </x:c>
+      <x:c r="L7" s="44" t="str">
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
+      </x:c>
+      <x:c r="M7" s="44" t="str">
+        <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
+2026-10-09 Step 2: 18-table Drizzle schema implemented with bilingual fields, seven property types, sale/rent rules, explicit price visibility and separate non-superuser migration/read-only app roles. Isolated local development/test PostgreSQL configured; no shared service modified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="310" customHeight="1">
+      <x:c r="A8" s="44" t="str">
+        <x:v>B02</x:v>
+      </x:c>
+      <x:c r="B8" s="44" t="str">
+        <x:v>Step 2 · Database</x:v>
+      </x:c>
+      <x:c r="C8" s="44" t="str">
+        <x:v>Migrations, foreign keys, constraints and rollback procedure</x:v>
+      </x:c>
+      <x:c r="D8" s="44" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="E8" s="44" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F8" s="44" t="str">
+        <x:v>Generated foundation and custom relational migrations, journal/snapshots, constraints/FKs/triggers and guarded test-only initial rollback implemented. Real pg_dump/committed rollback/pg_restore/rerun pass. No production migration performed.</x:v>
+      </x:c>
+      <x:c r="G8" s="44" t="str">
+        <x:v>Codex: generate reviewed additive migrations for later changes; production migration requires authorization and verified backup.</x:v>
+      </x:c>
+      <x:c r="H8" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I8" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J8" s="44" t="str">
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+      <x:c r="K8" s="44" t="str">
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
+      </x:c>
+      <x:c r="L8" s="44" t="str">
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
+      </x:c>
+      <x:c r="M8" s="44" t="str">
+        <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
+2026-10-09 Step 2: Generated foundation and custom relational migrations, journal/snapshots, constraints/FKs/triggers and guarded test-only initial rollback implemented. Real pg_dump/committed rollback/pg_restore/rerun pass. No production migration performed. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="310" customHeight="1">
+      <x:c r="A9" s="44" t="str">
+        <x:v>B03</x:v>
+      </x:c>
+      <x:c r="B9" s="44" t="str">
+        <x:v>Step 2 · Demo</x:v>
+      </x:c>
+      <x:c r="C9" s="44" t="str">
+        <x:v>Clearly fictional seed listings, projects and agents</x:v>
+      </x:c>
+      <x:c r="D9" s="44" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="E9" s="44" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F9" s="44" t="str">
+        <x:v>Repeatable local-only seed: 14 explicitly fictional listings, seven types/both intents and related demo records. Invalid domains, disabled users/agents, closed enquiries and off alerts. Public projection excludes demo inventory; no real prices/agents advertised.</x:v>
+      </x:c>
+      <x:c r="G9" s="44" t="str">
+        <x:v>Codex: keep demo data labelled and excluded from genuine inventory; seed only named local dev/test databases.</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I9" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J9" s="44" t="str">
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+      <x:c r="K9" s="44" t="str">
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
+      </x:c>
+      <x:c r="L9" s="44" t="str">
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
+      </x:c>
+      <x:c r="M9" s="44" t="str">
+        <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
+2026-10-09 Step 2: Repeatable local-only seed: 14 explicitly fictional listings, seven types/both intents and related demo records. Invalid domains, disabled users/agents, closed enquiries and off alerts. Public projection excludes demo inventory; no real prices/agents advertised. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="310" customHeight="1">
+      <x:c r="A10" s="44" t="str">
+        <x:v>B04</x:v>
+      </x:c>
+      <x:c r="B10" s="44" t="str">
+        <x:v>Step 2 · Search</x:v>
+      </x:c>
+      <x:c r="C10" s="44" t="str">
+        <x:v>Indexes for status, intent, type, price, location and title</x:v>
+      </x:c>
+      <x:c r="D10" s="44" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="E10" s="44" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F10" s="44" t="str">
+        <x:v>Intent/type/status/price, location/status, bounding coordinates, publication/feed and bilingual simple-text indexes implemented. Catalog and EXPLAIN use checks pass. Tiny-seed plans prove indexes are usable, not production speed.</x:v>
+      </x:c>
+      <x:c r="G10" s="44" t="str">
+        <x:v>Codex: use parameterized typed queries in Step 3; profile against realistic volume during later QA.</x:v>
+      </x:c>
+      <x:c r="H10" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I10" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J10" s="44" t="str">
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+      <x:c r="K10" s="44" t="str">
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
+      </x:c>
+      <x:c r="L10" s="44" t="str">
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
+      </x:c>
+      <x:c r="M10" s="44" t="str">
+        <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
+2026-10-09 Step 2: Intent/type/status/price, location/status, bounding coordinates, publication/feed and bilingual simple-text indexes implemented. Catalog and EXPLAIN use checks pass. Tiny-seed plans prove indexes are usable, not production speed. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="44"/>
@@ -32244,7 +32337,15 @@
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="E6:E10">
+      <x:formula1>"Done,Pending,Not started"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58e460fd3323412f"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -32280,7 +32381,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
+        <x:v>2026-10-09: Step 2 verified PostgreSQL schema/seed. 81 permanent IDs: 5 Done, 16 Pending, 60 Not started. Preserve append-only history. Test servers stop afterward.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -32302,14 +32403,14 @@
       </x:c>
       <x:c r="D3" s="18" t="n">
         <x:f>COUNTA('Done'!A6:A500)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F3" s="18" t="n">
         <x:f>COUNTA('Pending'!A6:A500)</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
         <x:v>Not started</x:v>
@@ -32321,7 +32422,7 @@
       </x:c>
       <x:c r="G4" s="22" t="n">
         <x:f>COUNTA('Not started'!A6:A500)</x:f>
-        <x:v>64</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
@@ -32365,7 +32466,7 @@
         <x:v>History</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="250" customHeight="1">
+    <x:row r="6" ht="310" customHeight="1">
       <x:c r="A6" s="46" t="str">
         <x:v>F02</x:v>
       </x:c>
@@ -32382,10 +32483,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F6" s="44" t="str">
-        <x:v>Approved gold and all section 2 colour tokens implemented and checked in eight shell tests. Overall runtime gates remain pending.</x:v>
+        <x:v>Owner approves gold / blue / teal / coral accent: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G6" s="44" t="str">
-        <x:v>Codex: preserve approved colours; complete remaining runtime gates.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H6" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -32394,18 +32495,20 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J6" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K6" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L6" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M6" s="44" t="str">
         <x:v>Original planning evidence: BUILD-SPEC §12 #1: accent not finalized
 2026-10-09 owner update: Owner selected approved wireframe colours: default gold #f2a91a and associated V3 tokens. Choice recorded; implementation/runtime completion gates remain pending.
-2026-10-09 foundation: Approved gold and all section 2 colour tokens implemented and checked in eight shell tests. Overall runtime gates remain pending. Owner requested localhost closure; do not reopen automatically.</x:v>
+2026-10-09 foundation: Approved gold and all section 2 colour tokens implemented and checked in eight shell tests. Overall runtime gates remain pending. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Approved gold and all section 2 colour tokens implemented and checked in eight shell tests. Overall runtime gates remain pending. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Owner approves gold / blue / teal / coral accent: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="250" customHeight="1">
@@ -32509,7 +32612,7 @@
       <x:c r="L9" s="44"/>
       <x:c r="M9" s="44"/>
     </x:row>
-    <x:row r="10" ht="200" customHeight="1">
+    <x:row r="10" ht="310" customHeight="1">
       <x:c r="A10" s="46" t="str">
         <x:v>B09</x:v>
       </x:c>
@@ -32517,7 +32620,7 @@
         <x:v>Decision · Map</x:v>
       </x:c>
       <x:c r="C10" s="44" t="str">
-        <x:v>Approve Google Maps Platform or Longdo Map</x:v>
+        <x:v>Select free open-source map library, tile/nearby provider and usage policy</x:v>
       </x:c>
       <x:c r="D10" s="44" t="str">
         <x:v>Backend</x:v>
@@ -32526,27 +32629,30 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F10" s="44" t="str">
-        <x:v>Owner requests free open-source mapping for now. Specific library and tile/nearby provider remain undecided.</x:v>
+        <x:v>Owner/V5 require free open-source mapping. Concrete provider/library/policy remain unresolved; Step 2 makes no choice.</x:v>
       </x:c>
       <x:c r="G10" s="44" t="str">
-        <x:v>Codex: evaluate free open-source mapping before map step; confirm provider and usage policy.</x:v>
-      </x:c>
-      <x:c r="H10" s="45"/>
+        <x:v>Codex: present free options and wait for owner choice under Step 4 authorization.</x:v>
+      </x:c>
+      <x:c r="H10" s="45" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="I10" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J10" s="44" t="str">
-        <x:v>Documentation-only update. Tracker/source-hash/mirror checks performed. No UI/backend code changed. Real-app/DB tests not run; components absent.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K10" s="44" t="str">
-        <x:v>Preceding verification commit c600068 pushed. Decision update will be committed and verified; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L10" s="44" t="str">
-        <x:v>Git/live matched before update. Changed documentation and canonical workbook mirrored only after divergence checks; final SHA-256 comparison required.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M10" s="44" t="str">
         <x:v>Original planning evidence: BUILD-SPEC §12 #8: map provider not selected
-2026-10-09 owner update: Owner requests free open-source mapping for now. Specific library and tile/nearby provider remain undecided.</x:v>
+2026-10-09 owner update: Owner requests free open-source mapping for now. Specific library and tile/nearby provider remain undecided.
+2026-10-09 Step 2: Owner/V5 require free open-source mapping. Concrete provider/library/policy remain unresolved; Step 2 makes no choice. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26" customHeight="1">
@@ -32730,7 +32836,7 @@
 2026-10-09 owner update: Owner selected both public and contact-gated pricing, chosen by admin per listing/product or project. Choice recorded; implementation pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="250" customHeight="1">
+    <x:row r="16" ht="310" customHeight="1">
       <x:c r="A16" s="44" t="str">
         <x:v>R01</x:v>
       </x:c>
@@ -32747,10 +32853,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F16" s="44" t="str">
-        <x:v>V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.</x:v>
+        <x:v>Step 2 schema/seed/runtime tests pass. Preparation closeout remains separate: V5 Step 0 tracker-update utility is not in the project and original local prototype rendering is browser-policy blocked. No duplicate IDs or source changes. Servers stop under latest request.</x:v>
       </x:c>
       <x:c r="G16" s="44" t="str">
-        <x:v>Owner: supply the next stage prompt or authorize deferred tests. Codex: follow V5 one stage at a time; do not automatically advance.</x:v>
+        <x:v>Codex: close the separate Step 0 utility/reference-review requirements only when authorized; stop before Step 3.</x:v>
       </x:c>
       <x:c r="H16" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -32759,23 +32865,24 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J16" s="44" t="str">
-        <x:v>Documentation/planning update only. No application tests run at owner request. Existing runtime test results remain in prior history. Workbook/source/mirror checks performed.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K16" s="44" t="str">
-        <x:v>Preceding foundation commit 604c62e pushed. V5 adoption commit/push verified at finalization; final report provides hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L16" s="44" t="str">
-        <x:v>Baseline live files compared with Git before synchronization; revised guide/source/docs/tracker synchronized only after divergence checks.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M16" s="44" t="str">
         <x:v>2026-10-09: Preparation recorded. Pending real-app/DB tests and localhost verification. Preserve this ID for subsequent updates.
 2026-10-09: cd897da pushed. Six sheets rendered; 81 IDs verified; 79 original IDs preserved. Preparation mirror hashes pass. R01 remains Pending for real-app/DB tests and localhost verification.
 2026-10-09 owner update: Owner choices documented and tracker updated. Foundation remains unbuilt; no app, PostgreSQL configuration or verified localhost URLs. Runtime gates remain pending.
 2026-10-09 foundation: Preparation and foundation implemented; docs/tracker/source mirror updated. Build passes; 12/16 browser/API tests passed before owner-requested closure. Four preference/search flows need retesting after fixes; PostgreSQL is unconfigured; port 3000 is closed. Owner requested localhost closure; do not reopen automatically.
-2026-10-09 V5 adoption: V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="250" customHeight="1">
+2026-10-09 V5 adoption: V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.
+2026-10-09 Step 2: Step 2 schema/seed/runtime tests pass. Preparation closeout remains separate: V5 Step 0 tracker-update utility is not in the project and original local prototype rendering is browser-policy blocked. No duplicate IDs or source changes. Servers stop under latest request. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="310" customHeight="1">
       <x:c r="A17" s="44" t="str">
         <x:v>F01</x:v>
       </x:c>
@@ -32792,10 +32899,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F17" s="44" t="str">
-        <x:v>Exact tokens, self-hosted fonts and reusable buttons/inputs/chips/tabs/dialogs/skeletons/search fields implemented. Final browser retests and real PostgreSQL completion gate remain pending.</x:v>
+        <x:v>Approved V3 CSS tokens, Prompt/Noto Sans Thai fonts, shared UI primitives: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G17" s="44" t="str">
-        <x:v>Codex: retest compiled final fixes when owner opens localhost; verify database gate.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H17" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -32804,20 +32911,22 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J17" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K17" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L17" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M17" s="44" t="str">
         <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
-2026-10-09 foundation: Exact tokens, self-hosted fonts and reusable buttons/inputs/chips/tabs/dialogs/skeletons/search fields implemented. Final browser retests and real PostgreSQL completion gate remain pending. Owner requested localhost closure; do not reopen automatically.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="250" customHeight="1">
+2026-10-09 foundation: Exact tokens, self-hosted fonts and reusable buttons/inputs/chips/tabs/dialogs/skeletons/search fields implemented. Final browser retests and real PostgreSQL completion gate remain pending. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Exact tokens, self-hosted fonts and reusable buttons/inputs/chips/tabs/dialogs/skeletons/search fields implemented. Final browser retests and real PostgreSQL completion gate remain pending. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Approved V3 CSS tokens, Prompt/Noto Sans Thai fonts, shared UI primitives: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="310" customHeight="1">
       <x:c r="A18" s="44" t="str">
         <x:v>F04</x:v>
       </x:c>
@@ -32834,10 +32943,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F18" s="44" t="str">
-        <x:v>Sticky 64px header, five desktop links, language/currency selector, Saved and rectangular Sign in implemented. All eight shell tests passed. Preference save fix needs retesting.</x:v>
+        <x:v>Sticky desktop header with one-line navigation and rectangular Sign in: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G18" s="44" t="str">
-        <x:v>Codex: retest preference flow when owner explicitly opens localhost.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H18" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -32846,20 +32955,22 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J18" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K18" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L18" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M18" s="44" t="str">
         <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
-2026-10-09 foundation: Sticky 64px header, five desktop links, language/currency selector, Saved and rectangular Sign in implemented. All eight shell tests passed. Preference save fix needs retesting. Owner requested localhost closure; do not reopen automatically.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="250" customHeight="1">
+2026-10-09 foundation: Sticky 64px header, five desktop links, language/currency selector, Saved and rectangular Sign in implemented. All eight shell tests passed. Preference save fix needs retesting. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Sticky 64px header, five desktop links, language/currency selector, Saved and rectangular Sign in implemented. All eight shell tests passed. Preference save fix needs retesting. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Sticky desktop header with one-line navigation and rectangular Sign in: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="310" customHeight="1">
       <x:c r="A19" s="44" t="str">
         <x:v>F05</x:v>
       </x:c>
@@ -32876,10 +32987,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F19" s="44" t="str">
-        <x:v>Responsive phone header and five safe-area bottom tabs implemented. 390px Thai/English shell tests passed. Final phone search containment change needs retesting.</x:v>
+        <x:v>Phone header, bottom tabs and responsive breakpoints: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G19" s="44" t="str">
-        <x:v>Codex: retest final phone search containment when localhost is opened.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H19" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -32888,20 +32999,22 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J19" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K19" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L19" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M19" s="44" t="str">
         <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
-2026-10-09 foundation: Responsive phone header and five safe-area bottom tabs implemented. 390px Thai/English shell tests passed. Final phone search containment change needs retesting. Owner requested localhost closure; do not reopen automatically.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="250" customHeight="1">
+2026-10-09 foundation: Responsive phone header and five safe-area bottom tabs implemented. 390px Thai/English shell tests passed. Final phone search containment change needs retesting. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Responsive phone header and five safe-area bottom tabs implemented. 390px Thai/English shell tests passed. Final phone search containment change needs retesting. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Phone header, bottom tabs and responsive breakpoints: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="310" customHeight="1">
       <x:c r="A20" s="44" t="str">
         <x:v>F06</x:v>
       </x:c>
@@ -32918,10 +33031,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F20" s="44" t="str">
-        <x:v>Approved soft-background footer with bilingual company/area/help links implemented. Actual LINE ID omitted until provided. Shell tests passed.</x:v>
+        <x:v>Light footer, company links, contact and PDPA link: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G20" s="44" t="str">
-        <x:v>Owner: supply contact details; Codex: complete runtime gates.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H20" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -32930,20 +33043,22 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J20" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K20" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L20" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M20" s="44" t="str">
         <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
-2026-10-09 foundation: Approved soft-background footer with bilingual company/area/help links implemented. Actual LINE ID omitted until provided. Shell tests passed. Owner requested localhost closure; do not reopen automatically.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="250" customHeight="1">
+2026-10-09 foundation: Approved soft-background footer with bilingual company/area/help links implemented. Actual LINE ID omitted until provided. Shell tests passed. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Approved soft-background footer with bilingual company/area/help links implemented. Actual LINE ID omitted until provided. Shell tests passed. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Light footer, company links, contact and PDPA link: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="310" customHeight="1">
       <x:c r="A21" s="44" t="str">
         <x:v>F07</x:v>
       </x:c>
@@ -32960,10 +33075,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F21" s="44" t="str">
-        <x:v>Thai/English routes, Accept-Language and explicit preference cookies implemented. Redirect checks passed. Four browser preference/search flows failed before closure; Host-based origin fix compiles but remains untested in browser.</x:v>
+        <x:v>Thai/English routes, language switch and localized formatting: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable.</x:v>
       </x:c>
       <x:c r="G21" s="44" t="str">
-        <x:v>Codex: rerun preference persistence and search tests when owner opens localhost.</x:v>
+        <x:v>Codex: preserve existing approved shell; any separate foundation closeout must use the latest passing evidence. Contact details remain owner-supplied.</x:v>
       </x:c>
       <x:c r="H21" s="45" t="d">
         <x:v>2026-10-09T00:00:00.000Z</x:v>
@@ -32972,60 +33087,35 @@
         <x:v>2026-10-09T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J21" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
+        <x:v>PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
       <x:c r="K21" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
+        <x:v>Preceding V5 commit 6e3d7d9 pushed. This Step 2 commit/push is verified during finalization; exact hash is in final report. If final push/sync fails, B01-B04/B34 must revert to Pending.</x:v>
       </x:c>
       <x:c r="L21" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
+        <x:v>44 baseline Git/live hashes matched before changes. Intended code/config/docs/tracker compared and synchronized; final SHA-256 check required before report. Credentials/runtime/deps/caches excluded.</x:v>
       </x:c>
       <x:c r="M21" s="44" t="str">
         <x:v>Original planning evidence: Not yet implemented; follow approved V3 handoff.
-2026-10-09 foundation: Thai/English routes, Accept-Language and explicit preference cookies implemented. Redirect checks passed. Four browser preference/search flows failed before closure; Host-based origin fix compiles but remains untested in browser. Owner requested localhost closure; do not reopen automatically.</x:v>
+2026-10-09 foundation: Thai/English routes, Accept-Language and explicit preference cookies implemented. Redirect checks passed. Four browser preference/search flows failed before closure; Host-based origin fix compiles but remains untested in browser. Owner requested localhost closure; do not reopen automatically.
+2026-10-09 Step 2: Thai/English routes, Accept-Language and explicit preference cookies implemented. Redirect checks passed. Four browser preference/search flows failed before closure; Host-based origin fix compiles but remains untested in browser. Latest evidence: all 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness verified. No Step 1 closeout or UI change is claimed in Step 2. Original prototype rendered comparison remains unverified. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
+2026-10-09 Step 2: Thai/English routes, language switch and localized formatting: implemented in the foundation. All 16 browser/API checks now pass, including the previous preference/search failures; real PostgreSQL readiness is verified. Pending separate foundation closeout: original rendered-prototype comparison remains unverified. Step 2 changes no UI. Owner contact details remain unresolved where applicable. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="250" customHeight="1">
-      <x:c r="A22" s="44" t="str">
-        <x:v>B34</x:v>
-      </x:c>
-      <x:c r="B22" s="44" t="str">
-        <x:v>Step 1 · Health</x:v>
-      </x:c>
-      <x:c r="C22" s="44" t="str">
-        <x:v>Basic /api/health endpoint with accurate application and database status</x:v>
-      </x:c>
-      <x:c r="D22" s="44" t="str">
-        <x:v>Backend</x:v>
-      </x:c>
-      <x:c r="E22" s="44" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="F22" s="44" t="str">
-        <x:v>Real health API implemented: HTTP 200 app ok, database not_configured, ready false before closure. Configured PostgreSQL is probed with Drizzle select 1; failure returns 503. No real database configuration exists.</x:v>
-      </x:c>
-      <x:c r="G22" s="44" t="str">
-        <x:v>Codex: verify against real PostgreSQL when configured and localhost opening is authorized.</x:v>
-      </x:c>
-      <x:c r="H22" s="45" t="d">
-        <x:v>2026-10-09T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="I22" s="45" t="d">
-        <x:v>2026-10-09T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="J22" s="44" t="str">
-        <x:v>PASS: final production build and TypeScript. Before closure: 12/16 Playwright tests (8 shell + 4 API/routing) at 390/768/1024/1440; 4 preference/search failures. Origin/phone fixes compile, browser retest pending. PostgreSQL not configured. Port 3000 closed on owner request.</x:v>
-      </x:c>
-      <x:c r="K22" s="44" t="str">
-        <x:v>Preceding owner-decisions commit 3f56908 pushed. Foundation commit/push verified at finalization; final report identifies its hash.</x:v>
-      </x:c>
-      <x:c r="L22" s="44" t="str">
-        <x:v>Baseline existing Git/live hashes matched. Intended foundation/docs/tracker safely synchronized and hash-checked at finalization; secrets/deps/caches excluded.</x:v>
-      </x:c>
-      <x:c r="M22" s="44" t="str">
-        <x:v>2026-10-09: Health API planned. No implementation in Step 0.
-2026-10-09 foundation: Real health API implemented: HTTP 200 app ok, database not_configured, ready false before closure. Configured PostgreSQL is probed with Drizzle select 1; failure returns 503. No real database configuration exists. Owner requested localhost closure; do not reopen automatically.</x:v>
-      </x:c>
+      <x:c r="A22" s="44"/>
+      <x:c r="B22" s="44"/>
+      <x:c r="C22" s="44"/>
+      <x:c r="D22" s="44"/>
+      <x:c r="E22" s="44"/>
+      <x:c r="F22" s="44"/>
+      <x:c r="G22" s="44"/>
+      <x:c r="H22" s="45"/>
+      <x:c r="I22" s="45"/>
+      <x:c r="J22" s="44"/>
+      <x:c r="K22" s="44"/>
+      <x:c r="L22" s="44"/>
+      <x:c r="M22" s="44"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="44"/>
@@ -40213,14 +40303,17 @@
       <x:formula>E6="Not started"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="E6:E22">
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="E22">
+      <x:formula1>"Done,Pending,Not started"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E6:E21">
       <x:formula1>"Done,Pending,Not started"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dcf99137e75432f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25f240809d04414e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40257,7 +40350,7 @@
     </x:row>
     <x:row r="2" ht="50" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>2026-10-09: Active V5 stage guide; owner-approved revised V3 references. No new build step or tests. 81 stable IDs; statuses unchanged. Preview open at owner request. Preserve append-only history.</x:v>
+        <x:v>2026-10-09: Step 2 verified PostgreSQL schema/seed. 81 permanent IDs: 5 Done, 16 Pending, 60 Not started. Preserve append-only history. Test servers stop afterward.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -40279,14 +40372,14 @@
       </x:c>
       <x:c r="D3" s="18" t="n">
         <x:f>COUNTA('Done'!A6:A500)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F3" s="18" t="n">
         <x:f>COUNTA('Pending'!A6:A500)</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G3" s="18" t="str">
         <x:v>Not started</x:v>
@@ -40298,7 +40391,7 @@
       </x:c>
       <x:c r="G4" s="22" t="n">
         <x:f>COUNTA('Not started'!A6:A500)</x:f>
-        <x:v>64</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
@@ -41218,13 +41311,13 @@
     </x:row>
     <x:row r="35" ht="26" customHeight="1">
       <x:c r="A35" s="46" t="str">
-        <x:v>B01</x:v>
+        <x:v>B05</x:v>
       </x:c>
       <x:c r="B35" s="44" t="str">
-        <x:v>Step 2 · Database</x:v>
+        <x:v>Step 2 · Filters</x:v>
       </x:c>
       <x:c r="C35" s="44" t="str">
-        <x:v>PostgreSQL/Drizzle schema for listings, projects, agents and users</x:v>
+        <x:v>Configurable filter-definition/option tables with safe allowed query fields</x:v>
       </x:c>
       <x:c r="D35" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41247,13 +41340,13 @@
     </x:row>
     <x:row r="36" ht="26" customHeight="1">
       <x:c r="A36" s="46" t="str">
-        <x:v>B02</x:v>
+        <x:v>B06</x:v>
       </x:c>
       <x:c r="B36" s="44" t="str">
-        <x:v>Step 2 · Database</x:v>
+        <x:v>Step 3 · Search</x:v>
       </x:c>
       <x:c r="C36" s="44" t="str">
-        <x:v>Migrations, foreign keys, constraints and rollback procedure</x:v>
+        <x:v>Typed validated listing/search data access and pagination</x:v>
       </x:c>
       <x:c r="D36" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41276,13 +41369,13 @@
     </x:row>
     <x:row r="37" ht="26" customHeight="1">
       <x:c r="A37" s="46" t="str">
-        <x:v>B03</x:v>
+        <x:v>B07</x:v>
       </x:c>
       <x:c r="B37" s="44" t="str">
-        <x:v>Step 2 · Demo</x:v>
+        <x:v>Step 3 · Search</x:v>
       </x:c>
       <x:c r="C37" s="44" t="str">
-        <x:v>Clearly fictional seed listings, projects and agents</x:v>
+        <x:v>Filter parsing, result counts, sort and histogram queries</x:v>
       </x:c>
       <x:c r="D37" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41305,13 +41398,13 @@
     </x:row>
     <x:row r="38" ht="26" customHeight="1">
       <x:c r="A38" s="46" t="str">
-        <x:v>B04</x:v>
+        <x:v>B08</x:v>
       </x:c>
       <x:c r="B38" s="44" t="str">
-        <x:v>Step 2 · Search</x:v>
+        <x:v>Step 4 · Map</x:v>
       </x:c>
       <x:c r="C38" s="44" t="str">
-        <x:v>Indexes for status, intent, type, price, location and title</x:v>
+        <x:v>Geospatial index, bounding-box search and hidden-pin privacy</x:v>
       </x:c>
       <x:c r="D38" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41334,13 +41427,13 @@
     </x:row>
     <x:row r="39" ht="26" customHeight="1">
       <x:c r="A39" s="46" t="str">
-        <x:v>B05</x:v>
+        <x:v>B10</x:v>
       </x:c>
       <x:c r="B39" s="44" t="str">
-        <x:v>Step 2 · Filters</x:v>
+        <x:v>Step 4 · Nearby</x:v>
       </x:c>
       <x:c r="C39" s="44" t="str">
-        <x:v>Configurable filter-definition/option tables with safe allowed query fields</x:v>
+        <x:v>Provider-backed nearby data ingest and 90-day refresh</x:v>
       </x:c>
       <x:c r="D39" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41363,13 +41456,13 @@
     </x:row>
     <x:row r="40" ht="26" customHeight="1">
       <x:c r="A40" s="46" t="str">
-        <x:v>B06</x:v>
+        <x:v>B11</x:v>
       </x:c>
       <x:c r="B40" s="44" t="str">
-        <x:v>Step 3 · Search</x:v>
+        <x:v>Step 5 · Media</x:v>
       </x:c>
       <x:c r="C40" s="44" t="str">
-        <x:v>Typed validated listing/search data access and pagination</x:v>
+        <x:v>Photo/floorplan/video metadata and safe image upload pipeline</x:v>
       </x:c>
       <x:c r="D40" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41392,13 +41485,13 @@
     </x:row>
     <x:row r="41" ht="26" customHeight="1">
       <x:c r="A41" s="46" t="str">
-        <x:v>B07</x:v>
+        <x:v>B12</x:v>
       </x:c>
       <x:c r="B41" s="44" t="str">
-        <x:v>Step 3 · Search</x:v>
+        <x:v>Step 5 · Similar</x:v>
       </x:c>
       <x:c r="C41" s="44" t="str">
-        <x:v>Filter parsing, result counts, sort and histogram queries</x:v>
+        <x:v>Same-location/type/intent matching with ±25% price fallback</x:v>
       </x:c>
       <x:c r="D41" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41421,13 +41514,13 @@
     </x:row>
     <x:row r="42" ht="26" customHeight="1">
       <x:c r="A42" s="46" t="str">
-        <x:v>B08</x:v>
+        <x:v>B13</x:v>
       </x:c>
       <x:c r="B42" s="44" t="str">
-        <x:v>Step 4 · Map</x:v>
+        <x:v>Step 5 · Metrics</x:v>
       </x:c>
       <x:c r="C42" s="44" t="str">
-        <x:v>Geospatial index, bounding-box search and hidden-pin privacy</x:v>
+        <x:v>Comparable pricing/yield gated by verified sample size</x:v>
       </x:c>
       <x:c r="D42" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41450,13 +41543,13 @@
     </x:row>
     <x:row r="43" ht="26" customHeight="1">
       <x:c r="A43" s="46" t="str">
-        <x:v>B10</x:v>
+        <x:v>B14</x:v>
       </x:c>
       <x:c r="B43" s="44" t="str">
-        <x:v>Step 4 · Nearby</x:v>
+        <x:v>Step 6 · Leads</x:v>
       </x:c>
       <x:c r="C43" s="44" t="str">
-        <x:v>Provider-backed nearby data ingest and 90-day refresh</x:v>
+        <x:v>Enquiry API validation and DB-first persist-before-notify flow</x:v>
       </x:c>
       <x:c r="D43" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41479,13 +41572,13 @@
     </x:row>
     <x:row r="44" ht="26" customHeight="1">
       <x:c r="A44" s="46" t="str">
-        <x:v>B11</x:v>
+        <x:v>B15</x:v>
       </x:c>
       <x:c r="B44" s="44" t="str">
-        <x:v>Step 5 · Media</x:v>
+        <x:v>Step 6 · Leads</x:v>
       </x:c>
       <x:c r="C44" s="44" t="str">
-        <x:v>Photo/floorplan/video metadata and safe image upload pipeline</x:v>
+        <x:v>PDPA consent version, UTM/source, language and audit metadata</x:v>
       </x:c>
       <x:c r="D44" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41508,13 +41601,13 @@
     </x:row>
     <x:row r="45" ht="26" customHeight="1">
       <x:c r="A45" s="46" t="str">
-        <x:v>B12</x:v>
+        <x:v>B16</x:v>
       </x:c>
       <x:c r="B45" s="44" t="str">
-        <x:v>Step 5 · Similar</x:v>
+        <x:v>Step 6 · Security</x:v>
       </x:c>
       <x:c r="C45" s="44" t="str">
-        <x:v>Same-location/type/intent matching with ±25% price fallback</x:v>
+        <x:v>Rate limits, honeypot and duplicate submission protection</x:v>
       </x:c>
       <x:c r="D45" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41537,13 +41630,13 @@
     </x:row>
     <x:row r="46" ht="26" customHeight="1">
       <x:c r="A46" s="46" t="str">
-        <x:v>B13</x:v>
+        <x:v>B19</x:v>
       </x:c>
       <x:c r="B46" s="44" t="str">
-        <x:v>Step 5 · Metrics</x:v>
+        <x:v>Step 6 · Chat</x:v>
       </x:c>
       <x:c r="C46" s="44" t="str">
-        <x:v>Comparable pricing/yield gated by verified sample size</x:v>
+        <x:v>Validated LINE/WhatsApp URLs and click event tracking</x:v>
       </x:c>
       <x:c r="D46" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41566,13 +41659,13 @@
     </x:row>
     <x:row r="47" ht="26" customHeight="1">
       <x:c r="A47" s="46" t="str">
-        <x:v>B14</x:v>
+        <x:v>B20</x:v>
       </x:c>
       <x:c r="B47" s="44" t="str">
-        <x:v>Step 6 · Leads</x:v>
+        <x:v>Step 8 · Projects</x:v>
       </x:c>
       <x:c r="C47" s="44" t="str">
-        <x:v>Enquiry API validation and DB-first persist-before-notify flow</x:v>
+        <x:v>Project/unit/plot status logic and validation</x:v>
       </x:c>
       <x:c r="D47" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41595,13 +41688,13 @@
     </x:row>
     <x:row r="48" ht="26" customHeight="1">
       <x:c r="A48" s="46" t="str">
-        <x:v>B15</x:v>
+        <x:v>B21</x:v>
       </x:c>
       <x:c r="B48" s="44" t="str">
-        <x:v>Step 6 · Leads</x:v>
+        <x:v>Step 8 · Booking</x:v>
       </x:c>
       <x:c r="C48" s="44" t="str">
-        <x:v>PDPA consent version, UTM/source, language and audit metadata</x:v>
+        <x:v>Site-visit availability and enquiry persistence, double-book protection</x:v>
       </x:c>
       <x:c r="D48" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41624,13 +41717,13 @@
     </x:row>
     <x:row r="49" ht="26" customHeight="1">
       <x:c r="A49" s="46" t="str">
-        <x:v>B16</x:v>
+        <x:v>B22</x:v>
       </x:c>
       <x:c r="B49" s="44" t="str">
-        <x:v>Step 6 · Security</x:v>
+        <x:v>Step 9 · Saved</x:v>
       </x:c>
       <x:c r="C49" s="44" t="str">
-        <x:v>Rate limits, honeypot and duplicate submission protection</x:v>
+        <x:v>Saved listings/searches persistence, new-match calculations</x:v>
       </x:c>
       <x:c r="D49" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41653,13 +41746,13 @@
     </x:row>
     <x:row r="50" ht="26" customHeight="1">
       <x:c r="A50" s="46" t="str">
-        <x:v>B19</x:v>
+        <x:v>B24</x:v>
       </x:c>
       <x:c r="B50" s="44" t="str">
-        <x:v>Step 6 · Chat</x:v>
+        <x:v>Step 10B · Auth</x:v>
       </x:c>
       <x:c r="C50" s="44" t="str">
-        <x:v>Validated LINE/WhatsApp URLs and click event tracking</x:v>
+        <x:v>Secure sessions, approved sign-in integrations and auth tests</x:v>
       </x:c>
       <x:c r="D50" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41682,13 +41775,13 @@
     </x:row>
     <x:row r="51" ht="26" customHeight="1">
       <x:c r="A51" s="46" t="str">
-        <x:v>B20</x:v>
+        <x:v>B25</x:v>
       </x:c>
       <x:c r="B51" s="44" t="str">
-        <x:v>Step 8 · Projects</x:v>
+        <x:v>Step 10B · Auth</x:v>
       </x:c>
       <x:c r="C51" s="44" t="str">
-        <x:v>Project/unit/plot status logic and validation</x:v>
+        <x:v>Account/localStorage saved-item merge and privacy isolation</x:v>
       </x:c>
       <x:c r="D51" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41711,13 +41804,13 @@
     </x:row>
     <x:row r="52" ht="26" customHeight="1">
       <x:c r="A52" s="46" t="str">
-        <x:v>B21</x:v>
+        <x:v>B26</x:v>
       </x:c>
       <x:c r="B52" s="44" t="str">
-        <x:v>Step 8 · Booking</x:v>
+        <x:v>Step 11B · Admin</x:v>
       </x:c>
       <x:c r="C52" s="44" t="str">
-        <x:v>Site-visit availability and enquiry persistence, double-book protection</x:v>
+        <x:v>Role-scoped CRUD for listings, images, projects, agents, filter config</x:v>
       </x:c>
       <x:c r="D52" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41740,13 +41833,13 @@
     </x:row>
     <x:row r="53" ht="26" customHeight="1">
       <x:c r="A53" s="46" t="str">
-        <x:v>B22</x:v>
+        <x:v>B27</x:v>
       </x:c>
       <x:c r="B53" s="44" t="str">
-        <x:v>Step 9 · Saved</x:v>
+        <x:v>Step 11B · Admin</x:v>
       </x:c>
       <x:c r="C53" s="44" t="str">
-        <x:v>Saved listings/searches persistence, new-match calculations</x:v>
+        <x:v>Admin user management, audit log and sensitive action authorization</x:v>
       </x:c>
       <x:c r="D53" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41769,13 +41862,13 @@
     </x:row>
     <x:row r="54" ht="26" customHeight="1">
       <x:c r="A54" s="46" t="str">
-        <x:v>B24</x:v>
+        <x:v>B30</x:v>
       </x:c>
       <x:c r="B54" s="44" t="str">
-        <x:v>Step 10B · Auth</x:v>
+        <x:v>Step 12 · Deploy</x:v>
       </x:c>
       <x:c r="C54" s="44" t="str">
-        <x:v>Secure sessions, approved sign-in integrations and auth tests</x:v>
+        <x:v>Single VPS deployment, TLS, backups and migration runbook</x:v>
       </x:c>
       <x:c r="D54" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41798,13 +41891,13 @@
     </x:row>
     <x:row r="55" ht="26" customHeight="1">
       <x:c r="A55" s="46" t="str">
-        <x:v>B25</x:v>
+        <x:v>B31</x:v>
       </x:c>
       <x:c r="B55" s="44" t="str">
-        <x:v>Step 10B · Auth</x:v>
+        <x:v>Step 12 · Quality</x:v>
       </x:c>
       <x:c r="C55" s="44" t="str">
-        <x:v>Account/localStorage saved-item merge and privacy isolation</x:v>
+        <x:v>Real PostgreSQL integration/Playwright tests and EXPLAIN ANALYZE</x:v>
       </x:c>
       <x:c r="D55" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41827,13 +41920,13 @@
     </x:row>
     <x:row r="56" ht="26" customHeight="1">
       <x:c r="A56" s="46" t="str">
-        <x:v>B26</x:v>
+        <x:v>B32</x:v>
       </x:c>
       <x:c r="B56" s="44" t="str">
-        <x:v>Step 11B · Admin</x:v>
+        <x:v>Step 12 · Security</x:v>
       </x:c>
       <x:c r="C56" s="44" t="str">
-        <x:v>Role-scoped CRUD for listings, images, projects, agents, filter config</x:v>
+        <x:v>Access control, PDPA, headers, secrets and rate-limit audit</x:v>
       </x:c>
       <x:c r="D56" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41856,13 +41949,13 @@
     </x:row>
     <x:row r="57" ht="26" customHeight="1">
       <x:c r="A57" s="46" t="str">
-        <x:v>B27</x:v>
+        <x:v>B33</x:v>
       </x:c>
       <x:c r="B57" s="44" t="str">
-        <x:v>Step 11B · Admin</x:v>
+        <x:v>Step 7 · Owners</x:v>
       </x:c>
       <x:c r="C57" s="44" t="str">
-        <x:v>Admin user management, audit log and sensitive action authorization</x:v>
+        <x:v>Home-value and service enquiry data handling</x:v>
       </x:c>
       <x:c r="D57" s="44" t="str">
         <x:v>Backend</x:v>
@@ -41885,16 +41978,16 @@
     </x:row>
     <x:row r="58" ht="26" customHeight="1">
       <x:c r="A58" s="46" t="str">
-        <x:v>B30</x:v>
+        <x:v>E01</x:v>
       </x:c>
       <x:c r="B58" s="44" t="str">
-        <x:v>Step 12 · Deploy</x:v>
+        <x:v>Step 6 · Email</x:v>
       </x:c>
       <x:c r="C58" s="44" t="str">
-        <x:v>Single VPS deployment, TLS, backups and migration runbook</x:v>
+        <x:v>Enquiry notification with retryable queue/outbox</x:v>
       </x:c>
       <x:c r="D58" s="44" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Email</x:v>
       </x:c>
       <x:c r="E58" s="44" t="str">
         <x:v>Not started</x:v>
@@ -41914,16 +42007,16 @@
     </x:row>
     <x:row r="59" ht="26" customHeight="1">
       <x:c r="A59" s="46" t="str">
-        <x:v>B31</x:v>
+        <x:v>E02</x:v>
       </x:c>
       <x:c r="B59" s="44" t="str">
-        <x:v>Step 12 · Quality</x:v>
+        <x:v>Step 6 · Email</x:v>
       </x:c>
       <x:c r="C59" s="44" t="str">
-        <x:v>Real PostgreSQL integration/Playwright tests and EXPLAIN ANALYZE</x:v>
+        <x:v>Thai and English buyer enquiry acknowledgments</x:v>
       </x:c>
       <x:c r="D59" s="44" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Email</x:v>
       </x:c>
       <x:c r="E59" s="44" t="str">
         <x:v>Not started</x:v>
@@ -41943,16 +42036,16 @@
     </x:row>
     <x:row r="60" ht="26" customHeight="1">
       <x:c r="A60" s="46" t="str">
-        <x:v>B32</x:v>
+        <x:v>E03</x:v>
       </x:c>
       <x:c r="B60" s="44" t="str">
-        <x:v>Step 12 · Security</x:v>
+        <x:v>Step 8 · Email</x:v>
       </x:c>
       <x:c r="C60" s="44" t="str">
-        <x:v>Access control, PDPA, headers, secrets and rate-limit audit</x:v>
+        <x:v>Project brochure/price list email delivery</x:v>
       </x:c>
       <x:c r="D60" s="44" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Email</x:v>
       </x:c>
       <x:c r="E60" s="44" t="str">
         <x:v>Not started</x:v>
@@ -41972,16 +42065,16 @@
     </x:row>
     <x:row r="61" ht="26" customHeight="1">
       <x:c r="A61" s="46" t="str">
-        <x:v>B33</x:v>
+        <x:v>E04</x:v>
       </x:c>
       <x:c r="B61" s="44" t="str">
-        <x:v>Step 7 · Owners</x:v>
+        <x:v>Step 8 · Email</x:v>
       </x:c>
       <x:c r="C61" s="44" t="str">
-        <x:v>Home-value and service enquiry data handling</x:v>
+        <x:v>Site visit request and confirmation notifications</x:v>
       </x:c>
       <x:c r="D61" s="44" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Email</x:v>
       </x:c>
       <x:c r="E61" s="44" t="str">
         <x:v>Not started</x:v>
@@ -42001,13 +42094,13 @@
     </x:row>
     <x:row r="62" ht="26" customHeight="1">
       <x:c r="A62" s="46" t="str">
-        <x:v>E01</x:v>
+        <x:v>E05</x:v>
       </x:c>
       <x:c r="B62" s="44" t="str">
-        <x:v>Step 6 · Email</x:v>
+        <x:v>Step 9 · Alerts</x:v>
       </x:c>
       <x:c r="C62" s="44" t="str">
-        <x:v>Enquiry notification with retryable queue/outbox</x:v>
+        <x:v>Instant/daily saved search email alerts for signed-in users</x:v>
       </x:c>
       <x:c r="D62" s="44" t="str">
         <x:v>Email</x:v>
@@ -42030,13 +42123,13 @@
     </x:row>
     <x:row r="63" ht="26" customHeight="1">
       <x:c r="A63" s="46" t="str">
-        <x:v>E02</x:v>
+        <x:v>E06</x:v>
       </x:c>
       <x:c r="B63" s="44" t="str">
-        <x:v>Step 6 · Email</x:v>
+        <x:v>Step 10B · Email</x:v>
       </x:c>
       <x:c r="C63" s="44" t="str">
-        <x:v>Thai and English buyer enquiry acknowledgments</x:v>
+        <x:v>Account verification and recovery messages if email auth approved</x:v>
       </x:c>
       <x:c r="D63" s="44" t="str">
         <x:v>Email</x:v>
@@ -42059,13 +42152,13 @@
     </x:row>
     <x:row r="64" ht="26" customHeight="1">
       <x:c r="A64" s="46" t="str">
-        <x:v>E03</x:v>
+        <x:v>E07</x:v>
       </x:c>
       <x:c r="B64" s="44" t="str">
-        <x:v>Step 8 · Email</x:v>
+        <x:v>Step 11B · Email</x:v>
       </x:c>
       <x:c r="C64" s="44" t="str">
-        <x:v>Project brochure/price list email delivery</x:v>
+        <x:v>Agent notification/routing administration</x:v>
       </x:c>
       <x:c r="D64" s="44" t="str">
         <x:v>Email</x:v>
@@ -42088,13 +42181,13 @@
     </x:row>
     <x:row r="65" ht="26" customHeight="1">
       <x:c r="A65" s="46" t="str">
-        <x:v>E04</x:v>
+        <x:v>E08</x:v>
       </x:c>
       <x:c r="B65" s="44" t="str">
-        <x:v>Step 8 · Email</x:v>
+        <x:v>Step 7 · Email</x:v>
       </x:c>
       <x:c r="C65" s="44" t="str">
-        <x:v>Site visit request and confirmation notifications</x:v>
+        <x:v>Home valuation and service enquiry replies</x:v>
       </x:c>
       <x:c r="D65" s="44" t="str">
         <x:v>Email</x:v>
@@ -42116,27 +42209,13 @@
       <x:c r="M65" s="44"/>
     </x:row>
     <x:row r="66" ht="26" customHeight="1">
-      <x:c r="A66" s="46" t="str">
-        <x:v>E05</x:v>
-      </x:c>
-      <x:c r="B66" s="44" t="str">
-        <x:v>Step 9 · Alerts</x:v>
-      </x:c>
-      <x:c r="C66" s="44" t="str">
-        <x:v>Instant/daily saved search email alerts for signed-in users</x:v>
-      </x:c>
-      <x:c r="D66" s="44" t="str">
-        <x:v>Email</x:v>
-      </x:c>
-      <x:c r="E66" s="44" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F66" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
-      </x:c>
-      <x:c r="G66" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
-      </x:c>
+      <x:c r="A66" s="46"/>
+      <x:c r="B66" s="44"/>
+      <x:c r="C66" s="44"/>
+      <x:c r="D66" s="44"/>
+      <x:c r="E66" s="44"/>
+      <x:c r="F66" s="44"/>
+      <x:c r="G66" s="44"/>
       <x:c r="H66" s="45"/>
       <x:c r="I66" s="45"/>
       <x:c r="J66" s="44"/>
@@ -42145,27 +42224,13 @@
       <x:c r="M66" s="44"/>
     </x:row>
     <x:row r="67" ht="26" customHeight="1">
-      <x:c r="A67" s="46" t="str">
-        <x:v>E06</x:v>
-      </x:c>
-      <x:c r="B67" s="44" t="str">
-        <x:v>Step 10B · Email</x:v>
-      </x:c>
-      <x:c r="C67" s="44" t="str">
-        <x:v>Account verification and recovery messages if email auth approved</x:v>
-      </x:c>
-      <x:c r="D67" s="44" t="str">
-        <x:v>Email</x:v>
-      </x:c>
-      <x:c r="E67" s="44" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F67" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
-      </x:c>
-      <x:c r="G67" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
-      </x:c>
+      <x:c r="A67" s="46"/>
+      <x:c r="B67" s="44"/>
+      <x:c r="C67" s="44"/>
+      <x:c r="D67" s="44"/>
+      <x:c r="E67" s="44"/>
+      <x:c r="F67" s="44"/>
+      <x:c r="G67" s="44"/>
       <x:c r="H67" s="45"/>
       <x:c r="I67" s="45"/>
       <x:c r="J67" s="44"/>
@@ -42174,27 +42239,13 @@
       <x:c r="M67" s="44"/>
     </x:row>
     <x:row r="68" ht="26" customHeight="1">
-      <x:c r="A68" s="46" t="str">
-        <x:v>E07</x:v>
-      </x:c>
-      <x:c r="B68" s="44" t="str">
-        <x:v>Step 11B · Email</x:v>
-      </x:c>
-      <x:c r="C68" s="44" t="str">
-        <x:v>Agent notification/routing administration</x:v>
-      </x:c>
-      <x:c r="D68" s="44" t="str">
-        <x:v>Email</x:v>
-      </x:c>
-      <x:c r="E68" s="44" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F68" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
-      </x:c>
-      <x:c r="G68" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
-      </x:c>
+      <x:c r="A68" s="46"/>
+      <x:c r="B68" s="44"/>
+      <x:c r="C68" s="44"/>
+      <x:c r="D68" s="44"/>
+      <x:c r="E68" s="44"/>
+      <x:c r="F68" s="44"/>
+      <x:c r="G68" s="44"/>
       <x:c r="H68" s="45"/>
       <x:c r="I68" s="45"/>
       <x:c r="J68" s="44"/>
@@ -42203,27 +42254,13 @@
       <x:c r="M68" s="44"/>
     </x:row>
     <x:row r="69" ht="26" customHeight="1">
-      <x:c r="A69" s="46" t="str">
-        <x:v>E08</x:v>
-      </x:c>
-      <x:c r="B69" s="44" t="str">
-        <x:v>Step 7 · Email</x:v>
-      </x:c>
-      <x:c r="C69" s="44" t="str">
-        <x:v>Home valuation and service enquiry replies</x:v>
-      </x:c>
-      <x:c r="D69" s="44" t="str">
-        <x:v>Email</x:v>
-      </x:c>
-      <x:c r="E69" s="44" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F69" s="44" t="str">
-        <x:v>Not yet implemented; follow approved V3 handoff.</x:v>
-      </x:c>
-      <x:c r="G69" s="44" t="str">
-        <x:v>Codex: implement in assigned step</x:v>
-      </x:c>
+      <x:c r="A69" s="46"/>
+      <x:c r="B69" s="44"/>
+      <x:c r="C69" s="44"/>
+      <x:c r="D69" s="44"/>
+      <x:c r="E69" s="44"/>
+      <x:c r="F69" s="44"/>
+      <x:c r="G69" s="44"/>
       <x:c r="H69" s="45"/>
       <x:c r="I69" s="45"/>
       <x:c r="J69" s="44"/>
@@ -48712,17 +48749,20 @@
       <x:formula>E6="Not started"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="E70:E75">
       <x:formula1>"Done,Pending,Not started"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="E6:E69">
+    <x:dataValidation type="list" sqref="E66:E69">
+      <x:formula1>"Done,Pending,Not started"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E6:E65">
       <x:formula1>"Done,Pending,Not started"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd923c45a72a64d84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22c0e574be984312"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Claude project handoff and current state
</commit_message>
<xml_diff>
--- a/Mstar-Property-Task-Tracker.xlsx
+++ b/Mstar-Property-Task-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="1" r:id="R27626f1841ef4132"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="2" r:id="R1b22002ff2cb479e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" r:id="R0989bca6f4704ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Done" sheetId="4" r:id="Rbffd9243c811433b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="5" r:id="Re71fca11b8984ef5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not started" sheetId="6" r:id="R19c5979771d742c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="1" r:id="R7b1e58856b4f4dde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="2" r:id="R994730cfbb2f457f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" r:id="R3390228af212415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Done" sheetId="4" r:id="Ra6e38bd544964f31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="5" r:id="R557ca3424aab4f96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not started" sheetId="6" r:id="R2cd2d7eda59d4a25"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -430,7 +430,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -440,7 +440,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -450,7 +450,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFF6666"/>
         </x:patternFill>
       </x:fill>
@@ -460,7 +460,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -470,7 +470,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -480,7 +480,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFF6666"/>
         </x:patternFill>
       </x:fill>
@@ -490,7 +490,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -500,7 +500,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -510,7 +510,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFF6666"/>
         </x:patternFill>
       </x:fill>
@@ -520,7 +520,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -530,7 +530,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -540,7 +540,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFF6666"/>
         </x:patternFill>
       </x:fill>
@@ -550,7 +550,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -560,7 +560,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -570,7 +570,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFF6666"/>
         </x:patternFill>
       </x:fill>
@@ -580,7 +580,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -590,7 +590,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -600,7 +600,7 @@
         <x:color rgb="FF000000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFF6666"/>
         </x:patternFill>
       </x:fill>
@@ -9164,7 +9164,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ee3b0fec5264935"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7e326bc49d5487a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9557,7 +9557,8 @@
 2026-10-09 foundation: Preparation and foundation implemented; docs/tracker/source mirror updated. Build passes; 12/16 browser/API tests passed before owner-requested closure. Four preference/search flows need retesting after fixes; PostgreSQL is unconfigured; port 3000 is closed. Owner requested localhost closure; do not reopen automatically.
 2026-10-09 V5 adoption: V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.
 2026-10-09 Step 2: Step 2 schema/seed/runtime tests pass. Preparation closeout remains separate: V5 Step 0 tracker-update utility is not in the project and original local prototype rendering is browser-policy blocked. No duplicate IDs or source changes. Servers stop under latest request. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
-2026-10-09 tracker formatting: workbook recreated with yellow Pending, light green Done and red Not started rows and status tabs. All 81 permanent IDs and prior task history preserved. Step 3 is authorized but implementation has not begun; owner requested the Excel first.</x:v>
+2026-10-09 tracker formatting: workbook recreated with yellow Pending, light green Done and red Not started rows and status tabs. All 81 permanent IDs and prior task history preserved. Step 3 is authorized but implementation has not begun; owner requested the Excel first.
+2026-10-09 Claude handoff: owner requested CLAUDE.md to share the current project context with Claude. Documented sources, Git/live paths, implemented shell/Step 2, unimplemented authorized Step 3, open decisions, safety, tests, servers and completion gates. Documentation/link checks and workbook ID/history/colour checks pass. No application change or new runtime test is claimed. R01 remains Pending for existing Step 0 blockers; Git/live synchronization and push are verified during finalization.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="26" customHeight="1">
@@ -17228,7 +17229,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03129b46c54d4819"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2317a333e2f4812"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24913,7 +24914,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eeb83cef3334d68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R585041451a67453f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32622,7 +32623,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R495b54da53904d6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfeedefc58826454b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33161,7 +33162,8 @@
 2026-10-09 foundation: Preparation and foundation implemented; docs/tracker/source mirror updated. Build passes; 12/16 browser/API tests passed before owner-requested closure. Four preference/search flows need retesting after fixes; PostgreSQL is unconfigured; port 3000 is closed. Owner requested localhost closure; do not reopen automatically.
 2026-10-09 V5 adoption: V5 adopted as active stage guide; updated owner-supplied V3 references preserved. No new application step started. Existing foundation Pending: browser tests deferred by owner; PostgreSQL unconfigured. Preview is open at owner request.
 2026-10-09 Step 2: Step 2 schema/seed/runtime tests pass. Preparation closeout remains separate: V5 Step 0 tracker-update utility is not in the project and original local prototype rendering is browser-policy blocked. No duplicate IDs or source changes. Servers stop under latest request. PASS: real PostgreSQL 18.6, 12/12 DB groups (migrations/rerun, fictional seed/rerun, insert/readback, joins, constraints/FKs, filter scope, indexes/EXPLAIN, privacy/permissions, pg_dump, committed rollback/restore). PASS: build/TypeScript, 16/16 Playwright at 390/768/1024/1440 in TH/EN. Real health 200/ready true, stopped DB 503, recovered 200. No implemented forms/admin; no form-delivery claim. Servers stop after task. Full npm audit: zero findings.
-2026-10-09 tracker formatting: workbook recreated with yellow Pending, light green Done and red Not started rows and status tabs. All 81 permanent IDs and prior task history preserved. Step 3 is authorized but implementation has not begun; owner requested the Excel first.</x:v>
+2026-10-09 tracker formatting: workbook recreated with yellow Pending, light green Done and red Not started rows and status tabs. All 81 permanent IDs and prior task history preserved. Step 3 is authorized but implementation has not begun; owner requested the Excel first.
+2026-10-09 Claude handoff: owner requested CLAUDE.md to share the current project context with Claude. Documented sources, Git/live paths, implemented shell/Step 2, unimplemented authorized Step 3, open decisions, safety, tests, servers and completion gates. Documentation/link checks and workbook ID/history/colour checks pass. No application change or new runtime test is claimed. R01 remains Pending for existing Step 0 blockers; Git/live synchronization and push are verified during finalization.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="310" customHeight="1">
@@ -40595,7 +40597,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabe72850259a4b3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re737f28ca1634620"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -49047,7 +49049,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4207507c36da4d49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67d3535895ac4ce3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>